<commit_message>
feat: initialize sub-process traceability system with build automation and label generation tools
</commit_message>
<xml_diff>
--- a/data/production_data.xlsx
+++ b/data/production_data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sub-process fill by TL" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,8 +54,8 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -63,49 +63,44 @@
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
+      <name val="Segoe UI"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
+      <b val="1"/>
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
-      <b val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
       <name val="Calibri"/>
       <color rgb="00000000"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -137,7 +132,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="29">
     <fill>
       <patternFill/>
     </fill>
@@ -230,8 +225,44 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF1B232C"/>
         <bgColor rgb="FF1B232C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0078D7"/>
+        <bgColor rgb="FF0078D7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF28A745"/>
+        <bgColor rgb="FF28A745"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -271,7 +302,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -311,13 +342,13 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
         <color auto="1"/>
@@ -326,10 +357,36 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
       </right>
       <top/>
       <bottom style="thin">
@@ -378,30 +435,15 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -411,6 +453,21 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -431,6 +488,19 @@
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -464,7 +534,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -478,105 +548,140 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="22" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="19" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="24" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="25" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="26" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="28" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -944,28 +1049,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:Q52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="7"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="11"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="13"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="25" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" style="27" min="1" max="1"/>
+    <col width="22" customWidth="1" style="27" min="2" max="2"/>
+    <col width="25" customWidth="1" style="27" min="3" max="3"/>
+    <col width="22" customWidth="1" style="27" min="4" max="4"/>
+    <col width="25" customWidth="1" style="27" min="5" max="7"/>
+    <col width="12" customWidth="1" style="27" min="6" max="6"/>
+    <col width="12" customWidth="1" style="27" min="7" max="7"/>
+    <col width="12" customWidth="1" style="27" min="8" max="8"/>
+    <col width="10" customWidth="1" style="27" min="9" max="9"/>
+    <col width="15" customWidth="1" style="27" min="10" max="11"/>
+    <col width="10" customWidth="1" style="27" min="11" max="11"/>
+    <col width="10" customWidth="1" style="27" min="12" max="13"/>
+    <col width="20" customWidth="1" style="27" min="13" max="13"/>
+    <col width="20" customWidth="1" style="27" min="14" max="14"/>
+    <col width="15" customWidth="1" style="27" min="15" max="15"/>
+    <col width="25" customWidth="1" style="27" min="16" max="16"/>
+    <col width="15" customWidth="1" style="27" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="34" customHeight="1" s="27">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>FULL PN° Semi fini</t>
@@ -1046,14 +1152,19 @@
           <t>Registered by ID</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="18.75" customHeight="1">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="Q1" s="33" t="inlineStr">
+        <is>
+          <t>Registered by ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18.75" customHeight="1" s="27">
+      <c r="A2" s="34" t="inlineStr">
         <is>
           <t>AT-V07-11313-A-SUB</t>
         </is>
       </c>
-      <c r="B2" s="25" t="inlineStr">
+      <c r="B2" s="34" t="inlineStr">
         <is>
           <t>SUB BODY N R</t>
         </is>
@@ -1068,64 +1179,64 @@
           <t>BODY R</t>
         </is>
       </c>
-      <c r="E2" s="26" t="inlineStr">
+      <c r="E2" s="35" t="inlineStr">
         <is>
           <t>TEST-123</t>
         </is>
       </c>
-      <c r="F2" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G2" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H2" s="26" t="n">
+      <c r="F2" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G2" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" s="35" t="n">
         <v>150</v>
       </c>
-      <c r="I2" s="26" t="inlineStr">
+      <c r="I2" s="35" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J2" s="26" t="inlineStr">
+      <c r="J2" s="35" t="inlineStr">
         <is>
           <t>888</t>
         </is>
       </c>
-      <c r="K2" s="26" t="inlineStr">
+      <c r="K2" s="35" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="L2" s="26" t="inlineStr">
+      <c r="L2" s="35" t="inlineStr">
         <is>
           <t>2026-06-07 18:07</t>
         </is>
       </c>
-      <c r="M2" s="26" t="inlineStr">
+      <c r="M2" s="35" t="inlineStr">
         <is>
           <t>2026-06-07 18:07</t>
         </is>
       </c>
-      <c r="N2" s="26" t="inlineStr">
+      <c r="N2" s="35" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="O2" s="26" t="inlineStr">
+      <c r="O2" s="35" t="inlineStr">
         <is>
           <t>Urgent order</t>
         </is>
       </c>
-      <c r="P2" s="22" t="n"/>
-    </row>
-    <row r="3" ht="18.75" customHeight="1">
-      <c r="A3" s="13" t="n"/>
-      <c r="B3" s="13" t="n"/>
+      <c r="P2" s="36" t="n"/>
+    </row>
+    <row r="3" ht="18.75" customHeight="1" s="27">
+      <c r="A3" s="18" t="n"/>
+      <c r="B3" s="18" t="n"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
           <t>AT-V07-11323-E-WIE</t>
@@ -1136,26 +1247,26 @@
           <t>BUMPER RUBBER R</t>
         </is>
       </c>
-      <c r="E3" s="13" t="n"/>
-      <c r="F3" s="13" t="n"/>
-      <c r="G3" s="13" t="n"/>
-      <c r="H3" s="13" t="n"/>
-      <c r="I3" s="13" t="n"/>
-      <c r="J3" s="13" t="n"/>
-      <c r="K3" s="13" t="n"/>
-      <c r="L3" s="13" t="n"/>
-      <c r="M3" s="13" t="n"/>
-      <c r="N3" s="13" t="n"/>
-      <c r="O3" s="13" t="n"/>
-      <c r="P3" s="23" t="n"/>
-    </row>
-    <row r="4" ht="18.75" customHeight="1">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="E3" s="18" t="n"/>
+      <c r="F3" s="18" t="n"/>
+      <c r="G3" s="18" t="n"/>
+      <c r="H3" s="18" t="n"/>
+      <c r="I3" s="18" t="n"/>
+      <c r="J3" s="18" t="n"/>
+      <c r="K3" s="18" t="n"/>
+      <c r="L3" s="18" t="n"/>
+      <c r="M3" s="18" t="n"/>
+      <c r="N3" s="18" t="n"/>
+      <c r="O3" s="18" t="n"/>
+      <c r="P3" s="37" t="n"/>
+    </row>
+    <row r="4" ht="18.75" customHeight="1" s="27">
+      <c r="A4" s="34" t="inlineStr">
         <is>
           <t>AT-V07-11314-A-SUB</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="34" t="inlineStr">
         <is>
           <t>SUB BODY N L</t>
         </is>
@@ -1170,68 +1281,68 @@
           <t>BODY L</t>
         </is>
       </c>
-      <c r="E4" s="26" t="inlineStr">
+      <c r="E4" s="35" t="inlineStr">
         <is>
           <t>HLAR568</t>
         </is>
       </c>
-      <c r="F4" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G4" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H4" s="26" t="n">
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" s="35" t="n">
         <v>120</v>
       </c>
-      <c r="I4" s="26" t="inlineStr">
+      <c r="I4" s="35" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="J4" s="26" t="inlineStr">
+      <c r="J4" s="35" t="inlineStr">
         <is>
           <t>567</t>
         </is>
       </c>
-      <c r="K4" s="26" t="inlineStr">
+      <c r="K4" s="35" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
       </c>
-      <c r="L4" s="26" t="inlineStr">
+      <c r="L4" s="35" t="inlineStr">
         <is>
           <t>2026-06-05 11:36</t>
         </is>
       </c>
-      <c r="M4" s="26" t="inlineStr">
+      <c r="M4" s="35" t="inlineStr">
         <is>
           <t>2026-06-07 18:32</t>
         </is>
       </c>
-      <c r="N4" s="26" t="inlineStr">
+      <c r="N4" s="35" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="O4" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P4" s="26" t="inlineStr">
+      <c r="O4" s="38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P4" s="35" t="inlineStr">
         <is>
           <t>543 / A</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18.75" customHeight="1">
-      <c r="A5" s="13" t="n"/>
-      <c r="B5" s="13" t="n"/>
+    <row r="5" ht="18.75" customHeight="1" s="27">
+      <c r="A5" s="18" t="n"/>
+      <c r="B5" s="18" t="n"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
           <t>AT-V07-11324-E-WIE</t>
@@ -1242,26 +1353,26 @@
           <t>BUMPER RUBBER L</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="13" t="n"/>
-      <c r="G5" s="13" t="n"/>
-      <c r="H5" s="13" t="n"/>
-      <c r="I5" s="13" t="n"/>
-      <c r="J5" s="13" t="n"/>
-      <c r="K5" s="13" t="n"/>
-      <c r="L5" s="13" t="n"/>
-      <c r="M5" s="13" t="n"/>
-      <c r="N5" s="13" t="n"/>
-      <c r="O5" s="13" t="n"/>
-      <c r="P5" s="13" t="n"/>
-    </row>
-    <row r="6" ht="18.75" customHeight="1">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
+      <c r="K5" s="18" t="n"/>
+      <c r="L5" s="18" t="n"/>
+      <c r="M5" s="18" t="n"/>
+      <c r="N5" s="18" t="n"/>
+      <c r="O5" s="37" t="n"/>
+      <c r="P5" s="18" t="n"/>
+    </row>
+    <row r="6" ht="18.75" customHeight="1" s="27">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>AT-V80-11311-A-SUB</t>
         </is>
       </c>
-      <c r="B6" s="25" t="inlineStr">
+      <c r="B6" s="34" t="inlineStr">
         <is>
           <t>Back plate R sub XDD</t>
         </is>
@@ -1276,68 +1387,68 @@
           <t>BACK PLATE (ZnNi) R</t>
         </is>
       </c>
-      <c r="E6" s="26" t="inlineStr">
+      <c r="E6" s="35" t="inlineStr">
         <is>
           <t>TEST12</t>
         </is>
       </c>
-      <c r="F6" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G6" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H6" s="26" t="n">
+      <c r="F6" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" s="35" t="n">
         <v>122</v>
       </c>
-      <c r="I6" s="26" t="inlineStr">
+      <c r="I6" s="35" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="J6" s="26" t="inlineStr">
+      <c r="J6" s="35" t="inlineStr">
         <is>
           <t>222</t>
         </is>
       </c>
-      <c r="K6" s="26" t="inlineStr">
+      <c r="K6" s="35" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="L6" s="26" t="inlineStr">
+      <c r="L6" s="35" t="inlineStr">
         <is>
           <t>2026-06-07 18:32</t>
         </is>
       </c>
-      <c r="M6" s="26" t="inlineStr">
+      <c r="M6" s="35" t="inlineStr">
         <is>
           <t>2026-06-07 18:33</t>
         </is>
       </c>
-      <c r="N6" s="26" t="inlineStr">
+      <c r="N6" s="35" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="O6" s="26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P6" s="26" t="inlineStr">
+      <c r="O6" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P6" s="35" t="inlineStr">
         <is>
           <t>543 / A</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="18.75" customHeight="1">
-      <c r="A7" s="13" t="n"/>
-      <c r="B7" s="13" t="n"/>
+    <row r="7" ht="18.75" customHeight="1" s="27">
+      <c r="A7" s="18" t="n"/>
+      <c r="B7" s="18" t="n"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
           <t>AT-V07-11359-B-WIE</t>
@@ -1348,26 +1459,26 @@
           <t>STOPPER RUBBER</t>
         </is>
       </c>
-      <c r="E7" s="13" t="n"/>
-      <c r="F7" s="13" t="n"/>
-      <c r="G7" s="13" t="n"/>
-      <c r="H7" s="13" t="n"/>
-      <c r="I7" s="13" t="n"/>
-      <c r="J7" s="13" t="n"/>
-      <c r="K7" s="13" t="n"/>
-      <c r="L7" s="13" t="n"/>
-      <c r="M7" s="13" t="n"/>
-      <c r="N7" s="13" t="n"/>
-      <c r="O7" s="13" t="n"/>
-      <c r="P7" s="13" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="18" t="n"/>
+      <c r="M7" s="18" t="n"/>
+      <c r="N7" s="18" t="n"/>
+      <c r="O7" s="18" t="n"/>
+      <c r="P7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="39" t="inlineStr">
         <is>
           <t>AT-V07-11214-A-SUB</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="39" t="inlineStr">
         <is>
           <t>SUB BODY EMG L</t>
         </is>
@@ -1382,68 +1493,68 @@
           <t>BODY(EMERGENCY) L</t>
         </is>
       </c>
-      <c r="E8" s="28" t="inlineStr">
+      <c r="E8" s="40" t="inlineStr">
         <is>
           <t>TEST2</t>
         </is>
       </c>
-      <c r="F8" s="28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H8" s="28" t="n">
+      <c r="F8" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="40" t="n">
         <v>22</v>
       </c>
-      <c r="I8" s="28" t="inlineStr">
+      <c r="I8" s="40" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="J8" s="28" t="inlineStr">
+      <c r="J8" s="40" t="inlineStr">
         <is>
           <t>323</t>
         </is>
       </c>
-      <c r="K8" s="28" t="inlineStr">
+      <c r="K8" s="40" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="L8" s="28" t="inlineStr">
+      <c r="L8" s="40" t="inlineStr">
         <is>
           <t>2026-06-06 13:39</t>
         </is>
       </c>
-      <c r="M8" s="28" t="inlineStr">
+      <c r="M8" s="40" t="inlineStr">
         <is>
           <t>2026-06-07 18:40</t>
         </is>
       </c>
-      <c r="N8" s="28" t="inlineStr">
+      <c r="N8" s="40" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="O8" s="28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P8" s="28" t="inlineStr">
+      <c r="O8" s="40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P8" s="40" t="inlineStr">
         <is>
           <t>567</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n"/>
-      <c r="B9" s="13" t="n"/>
+      <c r="A9" s="18" t="n"/>
+      <c r="B9" s="18" t="n"/>
       <c r="C9" s="4" t="inlineStr">
         <is>
           <t>AT-V07-11324-E-WIE</t>
@@ -1454,26 +1565,26 @@
           <t>BUMPER RUBBER L</t>
         </is>
       </c>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n"/>
-      <c r="G9" s="13" t="n"/>
-      <c r="H9" s="13" t="n"/>
-      <c r="I9" s="13" t="n"/>
-      <c r="J9" s="13" t="n"/>
-      <c r="K9" s="13" t="n"/>
-      <c r="L9" s="13" t="n"/>
-      <c r="M9" s="13" t="n"/>
-      <c r="N9" s="13" t="n"/>
-      <c r="O9" s="13" t="n"/>
-      <c r="P9" s="13" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
+      <c r="I9" s="18" t="n"/>
+      <c r="J9" s="18" t="n"/>
+      <c r="K9" s="18" t="n"/>
+      <c r="L9" s="18" t="n"/>
+      <c r="M9" s="18" t="n"/>
+      <c r="N9" s="18" t="n"/>
+      <c r="O9" s="18" t="n"/>
+      <c r="P9" s="18" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="41" t="inlineStr">
         <is>
           <t>AT-TEST-2026</t>
         </is>
       </c>
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="41" t="inlineStr">
         <is>
           <t>TEST PRODUCT</t>
         </is>
@@ -1488,68 +1599,68 @@
           <t>SPRING HOLDER</t>
         </is>
       </c>
-      <c r="E10" s="30" t="inlineStr">
+      <c r="E10" s="42" t="inlineStr">
         <is>
           <t>TESTPRD</t>
         </is>
       </c>
-      <c r="F10" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H10" s="30" t="n">
+      <c r="F10" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="42" t="n">
         <v>12</v>
       </c>
-      <c r="I10" s="30" t="inlineStr">
+      <c r="I10" s="42" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J10" s="30" t="inlineStr">
+      <c r="J10" s="42" t="inlineStr">
         <is>
           <t>122</t>
         </is>
       </c>
-      <c r="K10" s="30" t="inlineStr">
+      <c r="K10" s="42" t="inlineStr">
         <is>
           <t>S11</t>
         </is>
       </c>
-      <c r="L10" s="30" t="inlineStr">
+      <c r="L10" s="42" t="inlineStr">
         <is>
           <t>2026-06-07 18:55</t>
         </is>
       </c>
-      <c r="M10" s="30" t="inlineStr">
+      <c r="M10" s="42" t="inlineStr">
         <is>
           <t>2026-06-07 18:55</t>
         </is>
       </c>
-      <c r="N10" s="30" t="inlineStr">
+      <c r="N10" s="42" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="O10" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P10" s="30" t="inlineStr">
+      <c r="O10" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P10" s="42" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="n"/>
-      <c r="B11" s="20" t="n"/>
+      <c r="A11" s="17" t="n"/>
+      <c r="B11" s="17" t="n"/>
       <c r="C11" s="5" t="inlineStr">
         <is>
           <t>AT-TEST-2</t>
@@ -1560,22 +1671,22 @@
           <t>SPRING KEY</t>
         </is>
       </c>
-      <c r="E11" s="20" t="n"/>
-      <c r="F11" s="20" t="n"/>
-      <c r="G11" s="20" t="n"/>
-      <c r="H11" s="20" t="n"/>
-      <c r="I11" s="20" t="n"/>
-      <c r="J11" s="20" t="n"/>
-      <c r="K11" s="20" t="n"/>
-      <c r="L11" s="20" t="n"/>
-      <c r="M11" s="20" t="n"/>
-      <c r="N11" s="20" t="n"/>
-      <c r="O11" s="20" t="n"/>
-      <c r="P11" s="20" t="n"/>
+      <c r="E11" s="17" t="n"/>
+      <c r="F11" s="17" t="n"/>
+      <c r="G11" s="17" t="n"/>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="17" t="n"/>
+      <c r="J11" s="17" t="n"/>
+      <c r="K11" s="17" t="n"/>
+      <c r="L11" s="17" t="n"/>
+      <c r="M11" s="17" t="n"/>
+      <c r="N11" s="17" t="n"/>
+      <c r="O11" s="17" t="n"/>
+      <c r="P11" s="17" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="n"/>
-      <c r="B12" s="20" t="n"/>
+      <c r="A12" s="17" t="n"/>
+      <c r="B12" s="17" t="n"/>
       <c r="C12" s="5" t="inlineStr">
         <is>
           <t>AT-TEST-3</t>
@@ -1586,22 +1697,22 @@
           <t>ACCESS R</t>
         </is>
       </c>
-      <c r="E12" s="20" t="n"/>
-      <c r="F12" s="20" t="n"/>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="20" t="n"/>
-      <c r="I12" s="20" t="n"/>
-      <c r="J12" s="20" t="n"/>
-      <c r="K12" s="20" t="n"/>
-      <c r="L12" s="20" t="n"/>
-      <c r="M12" s="20" t="n"/>
-      <c r="N12" s="20" t="n"/>
-      <c r="O12" s="20" t="n"/>
-      <c r="P12" s="20" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="17" t="n"/>
+      <c r="H12" s="17" t="n"/>
+      <c r="I12" s="17" t="n"/>
+      <c r="J12" s="17" t="n"/>
+      <c r="K12" s="17" t="n"/>
+      <c r="L12" s="17" t="n"/>
+      <c r="M12" s="17" t="n"/>
+      <c r="N12" s="17" t="n"/>
+      <c r="O12" s="17" t="n"/>
+      <c r="P12" s="17" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="n"/>
-      <c r="B13" s="13" t="n"/>
+      <c r="A13" s="18" t="n"/>
+      <c r="B13" s="18" t="n"/>
       <c r="C13" s="5" t="inlineStr">
         <is>
           <t>AT-TEST-4</t>
@@ -1612,26 +1723,26 @@
           <t>PAWL</t>
         </is>
       </c>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="13" t="n"/>
-      <c r="H13" s="13" t="n"/>
-      <c r="I13" s="13" t="n"/>
-      <c r="J13" s="13" t="n"/>
-      <c r="K13" s="13" t="n"/>
-      <c r="L13" s="13" t="n"/>
-      <c r="M13" s="13" t="n"/>
-      <c r="N13" s="13" t="n"/>
-      <c r="O13" s="13" t="n"/>
-      <c r="P13" s="13" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="18" t="n"/>
+      <c r="H13" s="18" t="n"/>
+      <c r="I13" s="18" t="n"/>
+      <c r="J13" s="18" t="n"/>
+      <c r="K13" s="18" t="n"/>
+      <c r="L13" s="18" t="n"/>
+      <c r="M13" s="18" t="n"/>
+      <c r="N13" s="18" t="n"/>
+      <c r="O13" s="18" t="n"/>
+      <c r="P13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="41" t="inlineStr">
         <is>
           <t>AT-V07-11214-A-SUB</t>
         </is>
       </c>
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="41" t="inlineStr">
         <is>
           <t>SUB BODY EMG L</t>
         </is>
@@ -1646,68 +1757,68 @@
           <t>BODY(EMERGENCY) L</t>
         </is>
       </c>
-      <c r="E14" s="30" t="inlineStr">
+      <c r="E14" s="42" t="inlineStr">
         <is>
           <t>TATA</t>
         </is>
       </c>
-      <c r="F14" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" s="30" t="n">
+      <c r="F14" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="42" t="n">
         <v>112</v>
       </c>
-      <c r="I14" s="30" t="inlineStr">
+      <c r="I14" s="42" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="J14" s="30" t="inlineStr">
+      <c r="J14" s="42" t="inlineStr">
         <is>
           <t>222</t>
         </is>
       </c>
-      <c r="K14" s="30" t="inlineStr">
+      <c r="K14" s="42" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
       </c>
-      <c r="L14" s="30" t="inlineStr">
+      <c r="L14" s="42" t="inlineStr">
         <is>
           <t>2026-06-07 20:26</t>
         </is>
       </c>
-      <c r="M14" s="30" t="inlineStr">
+      <c r="M14" s="42" t="inlineStr">
         <is>
           <t>2026-06-08 15:55</t>
         </is>
       </c>
-      <c r="N14" s="30" t="inlineStr">
+      <c r="N14" s="42" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="O14" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P14" s="30" t="inlineStr">
+      <c r="O14" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P14" s="42" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="n"/>
-      <c r="B15" s="13" t="n"/>
+      <c r="A15" s="18" t="n"/>
+      <c r="B15" s="18" t="n"/>
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>AT-V07-11324-E-WIE</t>
@@ -1718,26 +1829,26 @@
           <t>BUMPER RUBBER L</t>
         </is>
       </c>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="13" t="n"/>
-      <c r="G15" s="13" t="n"/>
-      <c r="H15" s="13" t="n"/>
-      <c r="I15" s="13" t="n"/>
-      <c r="J15" s="13" t="n"/>
-      <c r="K15" s="13" t="n"/>
-      <c r="L15" s="13" t="n"/>
-      <c r="M15" s="13" t="n"/>
-      <c r="N15" s="13" t="n"/>
-      <c r="O15" s="13" t="n"/>
-      <c r="P15" s="13" t="n"/>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="18" t="n"/>
+      <c r="G15" s="18" t="n"/>
+      <c r="H15" s="18" t="n"/>
+      <c r="I15" s="18" t="n"/>
+      <c r="J15" s="18" t="n"/>
+      <c r="K15" s="18" t="n"/>
+      <c r="L15" s="18" t="n"/>
+      <c r="M15" s="18" t="n"/>
+      <c r="N15" s="18" t="n"/>
+      <c r="O15" s="18" t="n"/>
+      <c r="P15" s="18" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="41" t="inlineStr">
         <is>
           <t>MOCK-A01-10001-X-SUB</t>
         </is>
       </c>
-      <c r="B16" s="29" t="inlineStr">
+      <c r="B16" s="41" t="inlineStr">
         <is>
           <t>Alpha Subsystem Right</t>
         </is>
@@ -1752,68 +1863,68 @@
           <t>Alpha Core Right</t>
         </is>
       </c>
-      <c r="E16" s="30" t="inlineStr">
+      <c r="E16" s="42" t="inlineStr">
         <is>
           <t>HLAT</t>
         </is>
       </c>
-      <c r="F16" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G16" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H16" s="30" t="n">
+      <c r="F16" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G16" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" s="42" t="n">
         <v>120</v>
       </c>
-      <c r="I16" s="30" t="inlineStr">
+      <c r="I16" s="42" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J16" s="30" t="inlineStr">
+      <c r="J16" s="42" t="inlineStr">
         <is>
           <t>232</t>
         </is>
       </c>
-      <c r="K16" s="30" t="inlineStr">
+      <c r="K16" s="42" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="L16" s="30" t="inlineStr">
+      <c r="L16" s="42" t="inlineStr">
         <is>
           <t>2026-06-08 16:30</t>
         </is>
       </c>
-      <c r="M16" s="30" t="inlineStr">
+      <c r="M16" s="42" t="inlineStr">
         <is>
           <t>2026-06-08 16:31</t>
         </is>
       </c>
-      <c r="N16" s="30" t="inlineStr">
+      <c r="N16" s="42" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="O16" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P16" s="30" t="inlineStr">
+      <c r="O16" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P16" s="42" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="n"/>
-      <c r="B17" s="13" t="n"/>
+      <c r="A17" s="18" t="n"/>
+      <c r="B17" s="18" t="n"/>
       <c r="C17" s="5" t="inlineStr">
         <is>
           <t>MOCK-A01-10002-Z-PRT</t>
@@ -1824,26 +1935,26 @@
           <t>Alpha Buffer Right</t>
         </is>
       </c>
-      <c r="E17" s="13" t="n"/>
-      <c r="F17" s="13" t="n"/>
-      <c r="G17" s="13" t="n"/>
-      <c r="H17" s="13" t="n"/>
-      <c r="I17" s="13" t="n"/>
-      <c r="J17" s="13" t="n"/>
-      <c r="K17" s="13" t="n"/>
-      <c r="L17" s="13" t="n"/>
-      <c r="M17" s="13" t="n"/>
-      <c r="N17" s="13" t="n"/>
-      <c r="O17" s="13" t="n"/>
-      <c r="P17" s="13" t="n"/>
+      <c r="E17" s="18" t="n"/>
+      <c r="F17" s="18" t="n"/>
+      <c r="G17" s="18" t="n"/>
+      <c r="H17" s="18" t="n"/>
+      <c r="I17" s="18" t="n"/>
+      <c r="J17" s="18" t="n"/>
+      <c r="K17" s="18" t="n"/>
+      <c r="L17" s="18" t="n"/>
+      <c r="M17" s="18" t="n"/>
+      <c r="N17" s="18" t="n"/>
+      <c r="O17" s="18" t="n"/>
+      <c r="P17" s="18" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="41" t="inlineStr">
         <is>
           <t>MOCK-A01-10001-X-SUB</t>
         </is>
       </c>
-      <c r="B18" s="29" t="inlineStr">
+      <c r="B18" s="41" t="inlineStr">
         <is>
           <t>Alpha Subsystem Right</t>
         </is>
@@ -1858,68 +1969,68 @@
           <t>Alpha Core Right</t>
         </is>
       </c>
-      <c r="E18" s="30" t="inlineStr">
+      <c r="E18" s="42" t="inlineStr">
         <is>
           <t>HLAO</t>
         </is>
       </c>
-      <c r="F18" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G18" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H18" s="30" t="n">
+      <c r="F18" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="42" t="n">
         <v>120</v>
       </c>
-      <c r="I18" s="30" t="inlineStr">
+      <c r="I18" s="42" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="J18" s="30" t="inlineStr">
+      <c r="J18" s="42" t="inlineStr">
         <is>
           <t>888</t>
         </is>
       </c>
-      <c r="K18" s="30" t="inlineStr">
+      <c r="K18" s="42" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="L18" s="30" t="inlineStr">
+      <c r="L18" s="42" t="inlineStr">
         <is>
           <t>2026-06-08 16:39</t>
         </is>
       </c>
-      <c r="M18" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N18" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O18" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P18" s="30" t="inlineStr">
+      <c r="M18" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N18" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O18" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P18" s="42" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="n"/>
-      <c r="B19" s="13" t="n"/>
+      <c r="A19" s="18" t="n"/>
+      <c r="B19" s="18" t="n"/>
       <c r="C19" s="5" t="inlineStr">
         <is>
           <t>MOCK-A01-10002-Z-PRT</t>
@@ -1930,26 +2041,26 @@
           <t>Alpha Buffer Right</t>
         </is>
       </c>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="13" t="n"/>
-      <c r="G19" s="13" t="n"/>
-      <c r="H19" s="13" t="n"/>
-      <c r="I19" s="13" t="n"/>
-      <c r="J19" s="13" t="n"/>
-      <c r="K19" s="13" t="n"/>
-      <c r="L19" s="13" t="n"/>
-      <c r="M19" s="13" t="n"/>
-      <c r="N19" s="13" t="n"/>
-      <c r="O19" s="13" t="n"/>
-      <c r="P19" s="13" t="n"/>
+      <c r="E19" s="18" t="n"/>
+      <c r="F19" s="18" t="n"/>
+      <c r="G19" s="18" t="n"/>
+      <c r="H19" s="18" t="n"/>
+      <c r="I19" s="18" t="n"/>
+      <c r="J19" s="18" t="n"/>
+      <c r="K19" s="18" t="n"/>
+      <c r="L19" s="18" t="n"/>
+      <c r="M19" s="18" t="n"/>
+      <c r="N19" s="18" t="n"/>
+      <c r="O19" s="18" t="n"/>
+      <c r="P19" s="18" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="41" t="inlineStr">
         <is>
           <t>MOCK-A01-10001-X-SUB</t>
         </is>
       </c>
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="41" t="inlineStr">
         <is>
           <t>Alpha Subsystem Right</t>
         </is>
@@ -1964,68 +2075,68 @@
           <t>Alpha Core Right</t>
         </is>
       </c>
-      <c r="E20" s="30" t="inlineStr">
+      <c r="E20" s="42" t="inlineStr">
         <is>
           <t>HLAT</t>
         </is>
       </c>
-      <c r="F20" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="30" t="n">
+      <c r="F20" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="42" t="n">
         <v>123</v>
       </c>
-      <c r="I20" s="30" t="inlineStr">
+      <c r="I20" s="42" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="J20" s="30" t="inlineStr">
+      <c r="J20" s="42" t="inlineStr">
         <is>
           <t>333</t>
         </is>
       </c>
-      <c r="K20" s="30" t="inlineStr">
+      <c r="K20" s="42" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="L20" s="30" t="inlineStr">
+      <c r="L20" s="42" t="inlineStr">
         <is>
           <t>2026-06-08 17:40</t>
         </is>
       </c>
-      <c r="M20" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N20" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O20" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P20" s="30" t="inlineStr">
+      <c r="M20" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N20" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O20" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P20" s="42" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="n"/>
-      <c r="B21" s="13" t="n"/>
+      <c r="A21" s="18" t="n"/>
+      <c r="B21" s="18" t="n"/>
       <c r="C21" s="5" t="inlineStr">
         <is>
           <t>MOCK-A01-10002-Z-PRT</t>
@@ -2036,26 +2147,26 @@
           <t>Alpha Buffer Right</t>
         </is>
       </c>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="13" t="n"/>
-      <c r="G21" s="13" t="n"/>
-      <c r="H21" s="13" t="n"/>
-      <c r="I21" s="13" t="n"/>
-      <c r="J21" s="13" t="n"/>
-      <c r="K21" s="13" t="n"/>
-      <c r="L21" s="13" t="n"/>
-      <c r="M21" s="13" t="n"/>
-      <c r="N21" s="13" t="n"/>
-      <c r="O21" s="13" t="n"/>
-      <c r="P21" s="13" t="n"/>
+      <c r="E21" s="18" t="n"/>
+      <c r="F21" s="18" t="n"/>
+      <c r="G21" s="18" t="n"/>
+      <c r="H21" s="18" t="n"/>
+      <c r="I21" s="18" t="n"/>
+      <c r="J21" s="18" t="n"/>
+      <c r="K21" s="18" t="n"/>
+      <c r="L21" s="18" t="n"/>
+      <c r="M21" s="18" t="n"/>
+      <c r="N21" s="18" t="n"/>
+      <c r="O21" s="18" t="n"/>
+      <c r="P21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="29" t="inlineStr">
+      <c r="A22" s="41" t="inlineStr">
         <is>
           <t>MOCK-A01-10001-X-SUB</t>
         </is>
       </c>
-      <c r="B22" s="29" t="inlineStr">
+      <c r="B22" s="41" t="inlineStr">
         <is>
           <t>Alpha Subsystem Right</t>
         </is>
@@ -2070,68 +2181,68 @@
           <t>Alpha Core Right</t>
         </is>
       </c>
-      <c r="E22" s="30" t="inlineStr">
+      <c r="E22" s="42" t="inlineStr">
         <is>
           <t>HJKL</t>
         </is>
       </c>
-      <c r="F22" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G22" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H22" s="30" t="n">
+      <c r="F22" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="42" t="n">
         <v>333</v>
       </c>
-      <c r="I22" s="30" t="inlineStr">
+      <c r="I22" s="42" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J22" s="30" t="inlineStr">
+      <c r="J22" s="42" t="inlineStr">
         <is>
           <t>777</t>
         </is>
       </c>
-      <c r="K22" s="30" t="inlineStr">
+      <c r="K22" s="42" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
       </c>
-      <c r="L22" s="30" t="inlineStr">
+      <c r="L22" s="42" t="inlineStr">
         <is>
           <t>2026-06-08 17:41</t>
         </is>
       </c>
-      <c r="M22" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N22" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O22" s="30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P22" s="30" t="inlineStr">
+      <c r="M22" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N22" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O22" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P22" s="42" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="n"/>
-      <c r="B23" s="13" t="n"/>
+      <c r="A23" s="18" t="n"/>
+      <c r="B23" s="18" t="n"/>
       <c r="C23" s="5" t="inlineStr">
         <is>
           <t>MOCK-A01-10002-Z-PRT</t>
@@ -2142,1105 +2253,1745 @@
           <t>Alpha Buffer Right</t>
         </is>
       </c>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n"/>
-      <c r="G23" s="13" t="n"/>
-      <c r="H23" s="13" t="n"/>
-      <c r="I23" s="13" t="n"/>
-      <c r="J23" s="13" t="n"/>
-      <c r="K23" s="13" t="n"/>
-      <c r="L23" s="13" t="n"/>
-      <c r="M23" s="13" t="n"/>
-      <c r="N23" s="13" t="n"/>
-      <c r="O23" s="13" t="n"/>
-      <c r="P23" s="13" t="n"/>
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="18" t="n"/>
+      <c r="G23" s="18" t="n"/>
+      <c r="H23" s="18" t="n"/>
+      <c r="I23" s="18" t="n"/>
+      <c r="J23" s="18" t="n"/>
+      <c r="K23" s="18" t="n"/>
+      <c r="L23" s="18" t="n"/>
+      <c r="M23" s="18" t="n"/>
+      <c r="N23" s="18" t="n"/>
+      <c r="O23" s="18" t="n"/>
+      <c r="P23" s="18" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="43" t="inlineStr">
         <is>
           <t>MOCK-A01-10003-X-SUB</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B24" s="43" t="inlineStr">
         <is>
           <t>Alpha Subsystem Aux Right</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>MOCK-A01-10003-Y-PRT</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Alpha Core (Auxiliary) Right</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="44" t="inlineStr">
         <is>
           <t>RTR</t>
         </is>
       </c>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="12" t="n">
+      <c r="F24" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="44" t="n">
         <v>45</v>
       </c>
-      <c r="I24" s="12" t="inlineStr">
+      <c r="I24" s="44" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J24" s="12" t="inlineStr">
+      <c r="J24" s="44" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="K24" s="12" t="inlineStr">
+      <c r="K24" s="44" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="L24" s="12" t="inlineStr">
+      <c r="L24" s="44" t="inlineStr">
         <is>
           <t>2026-06-08 18:27</t>
         </is>
       </c>
-      <c r="M24" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N24" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O24" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P24" s="12" t="inlineStr">
+      <c r="M24" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N24" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O24" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P24" s="44" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n"/>
-      <c r="B25" s="13" t="n"/>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="A25" s="18" t="n"/>
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>MOCK-A01-10002-Z-PRT</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Alpha Buffer Right</t>
         </is>
       </c>
-      <c r="E25" s="13" t="n"/>
-      <c r="F25" s="13" t="n"/>
-      <c r="G25" s="13" t="n"/>
-      <c r="H25" s="13" t="n"/>
-      <c r="I25" s="13" t="n"/>
-      <c r="J25" s="13" t="n"/>
-      <c r="K25" s="13" t="n"/>
-      <c r="L25" s="13" t="n"/>
-      <c r="M25" s="13" t="n"/>
-      <c r="N25" s="13" t="n"/>
-      <c r="O25" s="13" t="n"/>
-      <c r="P25" s="13" t="n"/>
+      <c r="E25" s="18" t="n"/>
+      <c r="F25" s="18" t="n"/>
+      <c r="G25" s="18" t="n"/>
+      <c r="H25" s="18" t="n"/>
+      <c r="I25" s="18" t="n"/>
+      <c r="J25" s="18" t="n"/>
+      <c r="K25" s="18" t="n"/>
+      <c r="L25" s="18" t="n"/>
+      <c r="M25" s="18" t="n"/>
+      <c r="N25" s="18" t="n"/>
+      <c r="O25" s="18" t="n"/>
+      <c r="P25" s="18" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="43" t="inlineStr">
         <is>
           <t>MOCK-A01-10003-X-SUB</t>
         </is>
       </c>
-      <c r="B26" s="21" t="inlineStr">
+      <c r="B26" s="43" t="inlineStr">
         <is>
           <t>Alpha Subsystem Aux Right</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>MOCK-A01-10003-Y-PRT</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Alpha Core (Auxiliary) Right</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="44" t="inlineStr">
         <is>
           <t>TYTY</t>
         </is>
       </c>
-      <c r="F26" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H26" s="12" t="n">
+      <c r="F26" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="44" t="n">
         <v>23</v>
       </c>
-      <c r="I26" s="12" t="inlineStr">
+      <c r="I26" s="44" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J26" s="12" t="inlineStr">
+      <c r="J26" s="44" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="K26" s="12" t="inlineStr">
+      <c r="K26" s="44" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
       </c>
-      <c r="L26" s="12" t="inlineStr">
+      <c r="L26" s="44" t="inlineStr">
         <is>
           <t>2026-06-08 18:30</t>
         </is>
       </c>
-      <c r="M26" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O26" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P26" s="12" t="inlineStr">
+      <c r="M26" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N26" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O26" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P26" s="44" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="n"/>
-      <c r="B27" s="13" t="n"/>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="A27" s="18" t="n"/>
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>MOCK-A01-10002-Z-PRT</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Alpha Buffer Right</t>
         </is>
       </c>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n"/>
-      <c r="G27" s="13" t="n"/>
-      <c r="H27" s="13" t="n"/>
-      <c r="I27" s="13" t="n"/>
-      <c r="J27" s="13" t="n"/>
-      <c r="K27" s="13" t="n"/>
-      <c r="L27" s="13" t="n"/>
-      <c r="M27" s="13" t="n"/>
-      <c r="N27" s="13" t="n"/>
-      <c r="O27" s="13" t="n"/>
-      <c r="P27" s="13" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
+      <c r="G27" s="18" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="18" t="n"/>
+      <c r="J27" s="18" t="n"/>
+      <c r="K27" s="18" t="n"/>
+      <c r="L27" s="18" t="n"/>
+      <c r="M27" s="18" t="n"/>
+      <c r="N27" s="18" t="n"/>
+      <c r="O27" s="18" t="n"/>
+      <c r="P27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>MOCK-E05-50003-X-SUB</t>
         </is>
       </c>
-      <c r="B28" s="31" t="inlineStr">
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>Epsilon Housing Sub Left</t>
         </is>
       </c>
-      <c r="C28" s="32" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>MOCK-E05-50003-Y-PRT</t>
         </is>
       </c>
-      <c r="D28" s="32" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>Epsilon Housing Left</t>
         </is>
       </c>
-      <c r="E28" s="33" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>ERT</t>
         </is>
       </c>
-      <c r="F28" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G28" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H28" s="33" t="n">
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="n">
         <v>234</v>
       </c>
-      <c r="I28" s="33" t="inlineStr">
+      <c r="I28" s="16" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J28" s="33" t="inlineStr">
+      <c r="J28" s="16" t="inlineStr">
         <is>
           <t>233</t>
         </is>
       </c>
-      <c r="K28" s="33" t="inlineStr">
+      <c r="K28" s="16" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
       </c>
-      <c r="L28" s="33" t="inlineStr">
+      <c r="L28" s="16" t="inlineStr">
         <is>
           <t>2026-06-08 18:35</t>
         </is>
       </c>
-      <c r="M28" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N28" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O28" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P28" s="33" t="inlineStr">
+      <c r="M28" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N28" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O28" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P28" s="16" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="34" t="n"/>
-      <c r="B29" s="34" t="n"/>
-      <c r="C29" s="32" t="inlineStr">
+      <c r="A29" s="18" t="n"/>
+      <c r="B29" s="18" t="n"/>
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>MOCK-E05-50002-Z-PRT</t>
         </is>
       </c>
-      <c r="D29" s="32" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Epsilon Axis</t>
         </is>
       </c>
-      <c r="E29" s="34" t="n"/>
-      <c r="F29" s="34" t="n"/>
-      <c r="G29" s="34" t="n"/>
-      <c r="H29" s="34" t="n"/>
-      <c r="I29" s="34" t="n"/>
-      <c r="J29" s="34" t="n"/>
-      <c r="K29" s="34" t="n"/>
-      <c r="L29" s="34" t="n"/>
-      <c r="M29" s="34" t="n"/>
-      <c r="N29" s="34" t="n"/>
-      <c r="O29" s="34" t="n"/>
-      <c r="P29" s="34" t="n"/>
+      <c r="E29" s="18" t="n"/>
+      <c r="F29" s="18" t="n"/>
+      <c r="G29" s="18" t="n"/>
+      <c r="H29" s="18" t="n"/>
+      <c r="I29" s="18" t="n"/>
+      <c r="J29" s="18" t="n"/>
+      <c r="K29" s="18" t="n"/>
+      <c r="L29" s="18" t="n"/>
+      <c r="M29" s="18" t="n"/>
+      <c r="N29" s="18" t="n"/>
+      <c r="O29" s="18" t="n"/>
+      <c r="P29" s="18" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="31" t="inlineStr">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>MOCK-G07-70001-X-SUB</t>
         </is>
       </c>
-      <c r="B30" s="31" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>Omega Framework Sub Left</t>
         </is>
       </c>
-      <c r="C30" s="32" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>MOCK-G07-70001-Y-PRT</t>
         </is>
       </c>
-      <c r="D30" s="32" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Omega Anchor Left</t>
         </is>
       </c>
-      <c r="E30" s="33" t="inlineStr">
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>YUI</t>
         </is>
       </c>
-      <c r="F30" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G30" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H30" s="33" t="n">
+      <c r="F30" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G30" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="I30" s="33" t="inlineStr">
+      <c r="I30" s="16" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J30" s="33" t="inlineStr">
+      <c r="J30" s="16" t="inlineStr">
         <is>
           <t>778</t>
         </is>
       </c>
-      <c r="K30" s="33" t="inlineStr">
+      <c r="K30" s="16" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="L30" s="33" t="inlineStr">
+      <c r="L30" s="16" t="inlineStr">
         <is>
           <t>2026-06-08 18:39</t>
         </is>
       </c>
-      <c r="M30" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N30" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O30" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P30" s="33" t="inlineStr">
+      <c r="M30" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N30" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O30" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P30" s="16" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="39" t="n"/>
-      <c r="B31" s="39" t="n"/>
-      <c r="C31" s="32" t="inlineStr">
+      <c r="A31" s="17" t="n"/>
+      <c r="B31" s="17" t="n"/>
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>MOCK-G07-70002-Y-PRT</t>
         </is>
       </c>
-      <c r="D31" s="32" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Omega Frame Left</t>
         </is>
       </c>
-      <c r="E31" s="39" t="n"/>
-      <c r="F31" s="39" t="n"/>
-      <c r="G31" s="39" t="n"/>
-      <c r="H31" s="39" t="n"/>
-      <c r="I31" s="39" t="n"/>
-      <c r="J31" s="39" t="n"/>
-      <c r="K31" s="39" t="n"/>
-      <c r="L31" s="39" t="n"/>
-      <c r="M31" s="39" t="n"/>
-      <c r="N31" s="39" t="n"/>
-      <c r="O31" s="39" t="n"/>
-      <c r="P31" s="39" t="n"/>
+      <c r="E31" s="17" t="n"/>
+      <c r="F31" s="17" t="n"/>
+      <c r="G31" s="17" t="n"/>
+      <c r="H31" s="17" t="n"/>
+      <c r="I31" s="17" t="n"/>
+      <c r="J31" s="17" t="n"/>
+      <c r="K31" s="17" t="n"/>
+      <c r="L31" s="17" t="n"/>
+      <c r="M31" s="17" t="n"/>
+      <c r="N31" s="17" t="n"/>
+      <c r="O31" s="17" t="n"/>
+      <c r="P31" s="17" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="39" t="n"/>
-      <c r="B32" s="39" t="n"/>
-      <c r="C32" s="32" t="inlineStr">
+      <c r="A32" s="17" t="n"/>
+      <c r="B32" s="17" t="n"/>
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>MOCK-A01-10005-Z-PRT</t>
         </is>
       </c>
-      <c r="D32" s="32" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>Alpha Buffer Left</t>
         </is>
       </c>
-      <c r="E32" s="39" t="n"/>
-      <c r="F32" s="39" t="n"/>
-      <c r="G32" s="39" t="n"/>
-      <c r="H32" s="39" t="n"/>
-      <c r="I32" s="39" t="n"/>
-      <c r="J32" s="39" t="n"/>
-      <c r="K32" s="39" t="n"/>
-      <c r="L32" s="39" t="n"/>
-      <c r="M32" s="39" t="n"/>
-      <c r="N32" s="39" t="n"/>
-      <c r="O32" s="39" t="n"/>
-      <c r="P32" s="39" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17" t="n"/>
+      <c r="G32" s="17" t="n"/>
+      <c r="H32" s="17" t="n"/>
+      <c r="I32" s="17" t="n"/>
+      <c r="J32" s="17" t="n"/>
+      <c r="K32" s="17" t="n"/>
+      <c r="L32" s="17" t="n"/>
+      <c r="M32" s="17" t="n"/>
+      <c r="N32" s="17" t="n"/>
+      <c r="O32" s="17" t="n"/>
+      <c r="P32" s="17" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="34" t="n"/>
-      <c r="B33" s="34" t="n"/>
-      <c r="C33" s="32" t="inlineStr">
+      <c r="A33" s="18" t="n"/>
+      <c r="B33" s="18" t="n"/>
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>MOCK-B02-20002-Z-PRT</t>
         </is>
       </c>
-      <c r="D33" s="32" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>Beta Sealant</t>
         </is>
       </c>
-      <c r="E33" s="34" t="n"/>
-      <c r="F33" s="34" t="n"/>
-      <c r="G33" s="34" t="n"/>
-      <c r="H33" s="34" t="n"/>
-      <c r="I33" s="34" t="n"/>
-      <c r="J33" s="34" t="n"/>
-      <c r="K33" s="34" t="n"/>
-      <c r="L33" s="34" t="n"/>
-      <c r="M33" s="34" t="n"/>
-      <c r="N33" s="34" t="n"/>
-      <c r="O33" s="34" t="n"/>
-      <c r="P33" s="34" t="n"/>
+      <c r="E33" s="18" t="n"/>
+      <c r="F33" s="18" t="n"/>
+      <c r="G33" s="18" t="n"/>
+      <c r="H33" s="18" t="n"/>
+      <c r="I33" s="18" t="n"/>
+      <c r="J33" s="18" t="n"/>
+      <c r="K33" s="18" t="n"/>
+      <c r="L33" s="18" t="n"/>
+      <c r="M33" s="18" t="n"/>
+      <c r="N33" s="18" t="n"/>
+      <c r="O33" s="18" t="n"/>
+      <c r="P33" s="18" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="31" t="inlineStr">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t>MOCK-E05-50003-X-SUB</t>
         </is>
       </c>
-      <c r="B34" s="31" t="inlineStr">
+      <c r="B34" s="21" t="inlineStr">
         <is>
           <t>Epsilon Housing Sub Left</t>
         </is>
       </c>
-      <c r="C34" s="32" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>MOCK-E05-50003-Y-PRT</t>
         </is>
       </c>
-      <c r="D34" s="32" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>Epsilon Housing Left</t>
         </is>
       </c>
-      <c r="E34" s="33" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>TRS</t>
         </is>
       </c>
-      <c r="F34" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G34" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H34" s="33" t="n">
+      <c r="F34" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G34" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H34" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="I34" s="33" t="inlineStr">
+      <c r="I34" s="16" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J34" s="33" t="inlineStr">
+      <c r="J34" s="16" t="inlineStr">
         <is>
           <t>778</t>
         </is>
       </c>
-      <c r="K34" s="33" t="inlineStr">
+      <c r="K34" s="16" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="L34" s="33" t="inlineStr">
+      <c r="L34" s="16" t="inlineStr">
         <is>
           <t>2026-06-08 18:56</t>
         </is>
       </c>
-      <c r="M34" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N34" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O34" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P34" s="33" t="inlineStr">
+      <c r="M34" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N34" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O34" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P34" s="16" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="34" t="n"/>
-      <c r="B35" s="34" t="n"/>
-      <c r="C35" s="32" t="inlineStr">
+      <c r="A35" s="18" t="n"/>
+      <c r="B35" s="18" t="n"/>
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>MOCK-E05-50002-Z-PRT</t>
         </is>
       </c>
-      <c r="D35" s="32" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>Epsilon Axis</t>
         </is>
       </c>
-      <c r="E35" s="34" t="n"/>
-      <c r="F35" s="34" t="n"/>
-      <c r="G35" s="34" t="n"/>
-      <c r="H35" s="34" t="n"/>
-      <c r="I35" s="34" t="n"/>
-      <c r="J35" s="34" t="n"/>
-      <c r="K35" s="34" t="n"/>
-      <c r="L35" s="34" t="n"/>
-      <c r="M35" s="34" t="n"/>
-      <c r="N35" s="34" t="n"/>
-      <c r="O35" s="34" t="n"/>
-      <c r="P35" s="34" t="n"/>
+      <c r="E35" s="18" t="n"/>
+      <c r="F35" s="18" t="n"/>
+      <c r="G35" s="18" t="n"/>
+      <c r="H35" s="18" t="n"/>
+      <c r="I35" s="18" t="n"/>
+      <c r="J35" s="18" t="n"/>
+      <c r="K35" s="18" t="n"/>
+      <c r="L35" s="18" t="n"/>
+      <c r="M35" s="18" t="n"/>
+      <c r="N35" s="18" t="n"/>
+      <c r="O35" s="18" t="n"/>
+      <c r="P35" s="18" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="31" t="inlineStr">
+      <c r="A36" s="21" t="inlineStr">
         <is>
           <t>MOCK-B02-20004-X-SUB</t>
         </is>
       </c>
-      <c r="B36" s="31" t="inlineStr">
+      <c r="B36" s="21" t="inlineStr">
         <is>
           <t>Beta Panel Right Sub V2</t>
         </is>
       </c>
-      <c r="C36" s="32" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>MOCK-B02-20004-Y-PRT</t>
         </is>
       </c>
-      <c r="D36" s="32" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>Beta Panel (Upgraded) Right</t>
         </is>
       </c>
-      <c r="E36" s="33" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t>REE</t>
         </is>
       </c>
-      <c r="F36" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G36" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H36" s="33" t="n">
+      <c r="F36" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G36" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H36" s="16" t="n">
         <v>220</v>
       </c>
-      <c r="I36" s="33" t="inlineStr">
+      <c r="I36" s="16" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J36" s="33" t="inlineStr">
+      <c r="J36" s="16" t="inlineStr">
         <is>
           <t>778</t>
         </is>
       </c>
-      <c r="K36" s="33" t="inlineStr">
+      <c r="K36" s="16" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="L36" s="33" t="inlineStr">
+      <c r="L36" s="16" t="inlineStr">
         <is>
           <t>2026-06-08 18:58</t>
         </is>
       </c>
-      <c r="M36" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N36" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O36" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P36" s="33" t="inlineStr">
+      <c r="M36" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N36" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O36" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P36" s="16" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="34" t="n"/>
-      <c r="B37" s="34" t="n"/>
-      <c r="C37" s="32" t="inlineStr">
+      <c r="A37" s="18" t="n"/>
+      <c r="B37" s="18" t="n"/>
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>MOCK-B02-20002-Z-PRT</t>
         </is>
       </c>
-      <c r="D37" s="32" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>Beta Sealant</t>
         </is>
       </c>
-      <c r="E37" s="34" t="n"/>
-      <c r="F37" s="34" t="n"/>
-      <c r="G37" s="34" t="n"/>
-      <c r="H37" s="34" t="n"/>
-      <c r="I37" s="34" t="n"/>
-      <c r="J37" s="34" t="n"/>
-      <c r="K37" s="34" t="n"/>
-      <c r="L37" s="34" t="n"/>
-      <c r="M37" s="34" t="n"/>
-      <c r="N37" s="34" t="n"/>
-      <c r="O37" s="34" t="n"/>
-      <c r="P37" s="34" t="n"/>
+      <c r="E37" s="18" t="n"/>
+      <c r="F37" s="18" t="n"/>
+      <c r="G37" s="18" t="n"/>
+      <c r="H37" s="18" t="n"/>
+      <c r="I37" s="18" t="n"/>
+      <c r="J37" s="18" t="n"/>
+      <c r="K37" s="18" t="n"/>
+      <c r="L37" s="18" t="n"/>
+      <c r="M37" s="18" t="n"/>
+      <c r="N37" s="18" t="n"/>
+      <c r="O37" s="18" t="n"/>
+      <c r="P37" s="18" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="31" t="inlineStr">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t>MOCK-G07-70001-X-SUB</t>
         </is>
       </c>
-      <c r="B38" s="31" t="inlineStr">
+      <c r="B38" s="21" t="inlineStr">
         <is>
           <t>Omega Framework Sub Left</t>
         </is>
       </c>
-      <c r="C38" s="32" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>MOCK-G07-70001-Y-PRT</t>
         </is>
       </c>
-      <c r="D38" s="32" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
         <is>
           <t>Omega Anchor Left</t>
         </is>
       </c>
-      <c r="E38" s="33" t="inlineStr">
+      <c r="E38" s="16" t="inlineStr">
         <is>
           <t>FFG</t>
         </is>
       </c>
-      <c r="F38" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G38" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H38" s="33" t="n">
+      <c r="F38" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G38" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H38" s="16" t="n">
         <v>900</v>
       </c>
-      <c r="I38" s="33" t="inlineStr">
+      <c r="I38" s="16" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="J38" s="33" t="inlineStr">
+      <c r="J38" s="16" t="inlineStr">
         <is>
           <t>778</t>
         </is>
       </c>
-      <c r="K38" s="33" t="inlineStr">
+      <c r="K38" s="16" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="L38" s="33" t="inlineStr">
+      <c r="L38" s="16" t="inlineStr">
         <is>
           <t>2026-06-08 19:13</t>
         </is>
       </c>
-      <c r="M38" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N38" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O38" s="33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P38" s="33" t="inlineStr">
+      <c r="M38" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-09 17:06</t>
+        </is>
+      </c>
+      <c r="N38" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O38" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P38" s="16" t="inlineStr">
         <is>
           <t>999</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="39" t="n"/>
-      <c r="B39" s="39" t="n"/>
-      <c r="C39" s="32" t="inlineStr">
+      <c r="A39" s="17" t="n"/>
+      <c r="B39" s="17" t="n"/>
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>MOCK-G07-70002-Y-PRT</t>
         </is>
       </c>
-      <c r="D39" s="32" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t>Omega Frame Left</t>
         </is>
       </c>
-      <c r="E39" s="39" t="n"/>
-      <c r="F39" s="39" t="n"/>
-      <c r="G39" s="39" t="n"/>
-      <c r="H39" s="39" t="n"/>
-      <c r="I39" s="39" t="n"/>
-      <c r="J39" s="39" t="n"/>
-      <c r="K39" s="39" t="n"/>
-      <c r="L39" s="39" t="n"/>
-      <c r="M39" s="39" t="n"/>
-      <c r="N39" s="39" t="n"/>
-      <c r="O39" s="39" t="n"/>
-      <c r="P39" s="39" t="n"/>
+      <c r="E39" s="17" t="n"/>
+      <c r="F39" s="17" t="n"/>
+      <c r="G39" s="17" t="n"/>
+      <c r="H39" s="17" t="n"/>
+      <c r="I39" s="17" t="n"/>
+      <c r="J39" s="17" t="n"/>
+      <c r="K39" s="17" t="n"/>
+      <c r="L39" s="17" t="n"/>
+      <c r="M39" s="17" t="n"/>
+      <c r="N39" s="17" t="n"/>
+      <c r="O39" s="17" t="n"/>
+      <c r="P39" s="17" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="39" t="n"/>
-      <c r="B40" s="39" t="n"/>
-      <c r="C40" s="32" t="inlineStr">
+      <c r="A40" s="17" t="n"/>
+      <c r="B40" s="17" t="n"/>
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>MOCK-A01-10005-Z-PRT</t>
         </is>
       </c>
-      <c r="D40" s="32" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>Alpha Buffer Left</t>
         </is>
       </c>
-      <c r="E40" s="39" t="n"/>
-      <c r="F40" s="39" t="n"/>
-      <c r="G40" s="39" t="n"/>
-      <c r="H40" s="39" t="n"/>
-      <c r="I40" s="39" t="n"/>
-      <c r="J40" s="39" t="n"/>
-      <c r="K40" s="39" t="n"/>
-      <c r="L40" s="39" t="n"/>
-      <c r="M40" s="39" t="n"/>
-      <c r="N40" s="39" t="n"/>
-      <c r="O40" s="39" t="n"/>
-      <c r="P40" s="39" t="n"/>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="17" t="n"/>
+      <c r="G40" s="17" t="n"/>
+      <c r="H40" s="17" t="n"/>
+      <c r="I40" s="17" t="n"/>
+      <c r="J40" s="17" t="n"/>
+      <c r="K40" s="17" t="n"/>
+      <c r="L40" s="17" t="n"/>
+      <c r="M40" s="17" t="n"/>
+      <c r="N40" s="17" t="n"/>
+      <c r="O40" s="17" t="n"/>
+      <c r="P40" s="17" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="34" t="n"/>
-      <c r="B41" s="34" t="n"/>
-      <c r="C41" s="32" t="inlineStr">
+      <c r="A41" s="18" t="n"/>
+      <c r="B41" s="18" t="n"/>
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>MOCK-B02-20002-Z-PRT</t>
         </is>
       </c>
-      <c r="D41" s="32" t="inlineStr">
+      <c r="D41" s="7" t="inlineStr">
         <is>
           <t>Beta Sealant</t>
         </is>
       </c>
-      <c r="E41" s="34" t="n"/>
-      <c r="F41" s="34" t="n"/>
-      <c r="G41" s="34" t="n"/>
-      <c r="H41" s="34" t="n"/>
-      <c r="I41" s="34" t="n"/>
-      <c r="J41" s="34" t="n"/>
-      <c r="K41" s="34" t="n"/>
-      <c r="L41" s="34" t="n"/>
-      <c r="M41" s="34" t="n"/>
-      <c r="N41" s="34" t="n"/>
-      <c r="O41" s="34" t="n"/>
-      <c r="P41" s="34" t="n"/>
+      <c r="E41" s="18" t="n"/>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="18" t="n"/>
+      <c r="H41" s="18" t="n"/>
+      <c r="I41" s="18" t="n"/>
+      <c r="J41" s="18" t="n"/>
+      <c r="K41" s="18" t="n"/>
+      <c r="L41" s="18" t="n"/>
+      <c r="M41" s="18" t="n"/>
+      <c r="N41" s="18" t="n"/>
+      <c r="O41" s="18" t="n"/>
+      <c r="P41" s="18" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20001-X-SUB</t>
+        </is>
+      </c>
+      <c r="B42" s="21" t="inlineStr">
+        <is>
+          <t>Beta Panel Right Sub</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20001-Y-PRT</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Beta Panel Right</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>QT67</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G42" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H42" s="16" t="n">
+        <v>900</v>
+      </c>
+      <c r="I42" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J42" s="16" t="inlineStr">
+        <is>
+          <t>778</t>
+        </is>
+      </c>
+      <c r="K42" s="16" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="L42" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-09 16:05</t>
+        </is>
+      </c>
+      <c r="M42" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-09 16:17</t>
+        </is>
+      </c>
+      <c r="N42" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="O42" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P42" s="16" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="18" t="n"/>
+      <c r="B43" s="18" t="n"/>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Beta Sealant</t>
+        </is>
+      </c>
+      <c r="E43" s="18" t="n"/>
+      <c r="F43" s="18" t="n"/>
+      <c r="G43" s="18" t="n"/>
+      <c r="H43" s="18" t="n"/>
+      <c r="I43" s="18" t="n"/>
+      <c r="J43" s="18" t="n"/>
+      <c r="K43" s="18" t="n"/>
+      <c r="L43" s="18" t="n"/>
+      <c r="M43" s="18" t="n"/>
+      <c r="N43" s="18" t="n"/>
+      <c r="O43" s="18" t="n"/>
+      <c r="P43" s="18" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>MOCK-C03-30006-X-SUB</t>
+        </is>
+      </c>
+      <c r="B44" s="21" t="inlineStr">
+        <is>
+          <t>Gamma Switch Right Sub (Long)</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-C03-30006-Y-PRT</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Gamma Switch Long Right</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G44" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H44" s="16" t="n">
+        <v>90</v>
+      </c>
+      <c r="I44" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J44" s="16" t="inlineStr">
+        <is>
+          <t>770</t>
+        </is>
+      </c>
+      <c r="K44" s="16" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="L44" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-09 16:31</t>
+        </is>
+      </c>
+      <c r="M44" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N44" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O44" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P44" s="16" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="n"/>
+      <c r="B45" s="17" t="n"/>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-C03-30002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Gamma Coil Right</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="n"/>
+      <c r="F45" s="17" t="n"/>
+      <c r="G45" s="17" t="n"/>
+      <c r="H45" s="17" t="n"/>
+      <c r="I45" s="17" t="n"/>
+      <c r="J45" s="17" t="n"/>
+      <c r="K45" s="17" t="n"/>
+      <c r="L45" s="17" t="n"/>
+      <c r="M45" s="17" t="n"/>
+      <c r="N45" s="17" t="n"/>
+      <c r="O45" s="17" t="n"/>
+      <c r="P45" s="17" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="18" t="n"/>
+      <c r="B46" s="18" t="n"/>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-C03-30003-W-PRT</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Gamma Pin</t>
+        </is>
+      </c>
+      <c r="E46" s="18" t="n"/>
+      <c r="F46" s="18" t="n"/>
+      <c r="G46" s="18" t="n"/>
+      <c r="H46" s="18" t="n"/>
+      <c r="I46" s="18" t="n"/>
+      <c r="J46" s="18" t="n"/>
+      <c r="K46" s="18" t="n"/>
+      <c r="L46" s="18" t="n"/>
+      <c r="M46" s="18" t="n"/>
+      <c r="N46" s="18" t="n"/>
+      <c r="O46" s="18" t="n"/>
+      <c r="P46" s="18" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="21" t="inlineStr">
+        <is>
+          <t>MOCK-E05-50003-X-SUB</t>
+        </is>
+      </c>
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>Epsilon Housing Sub Left</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-E05-50003-Y-PRT</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Epsilon Housing Left</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>89456</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G47" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H47" s="16" t="n">
+        <v>134</v>
+      </c>
+      <c r="I47" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J47" s="16" t="inlineStr">
+        <is>
+          <t>771</t>
+        </is>
+      </c>
+      <c r="K47" s="16" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="L47" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-09 16:53</t>
+        </is>
+      </c>
+      <c r="M47" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N47" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O47" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P47" s="16" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="18" t="n"/>
+      <c r="B48" s="18" t="n"/>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-E05-50002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Epsilon Axis</t>
+        </is>
+      </c>
+      <c r="E48" s="18" t="n"/>
+      <c r="F48" s="18" t="n"/>
+      <c r="G48" s="18" t="n"/>
+      <c r="H48" s="18" t="n"/>
+      <c r="I48" s="18" t="n"/>
+      <c r="J48" s="18" t="n"/>
+      <c r="K48" s="18" t="n"/>
+      <c r="L48" s="18" t="n"/>
+      <c r="M48" s="18" t="n"/>
+      <c r="N48" s="18" t="n"/>
+      <c r="O48" s="18" t="n"/>
+      <c r="P48" s="18" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="45" t="inlineStr">
+        <is>
+          <t>SB202606091815S07C01</t>
+        </is>
+      </c>
+      <c r="B49" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10006-X-SUB</t>
+        </is>
+      </c>
+      <c r="C49" s="45" t="inlineStr">
+        <is>
+          <t>Alpha Subsystem Aux Left</t>
+        </is>
+      </c>
+      <c r="D49" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10006-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E49" s="46" t="inlineStr">
+        <is>
+          <t>Alpha Core (Auxiliary) Left</t>
+        </is>
+      </c>
+      <c r="F49" s="47" t="inlineStr">
+        <is>
+          <t>TRES</t>
+        </is>
+      </c>
+      <c r="G49" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H49" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I49" s="47" t="n">
+        <v>130</v>
+      </c>
+      <c r="J49" s="47" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="K49" s="47" t="inlineStr">
+        <is>
+          <t>543</t>
+        </is>
+      </c>
+      <c r="L49" s="47" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="M49" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09 18:15</t>
+        </is>
+      </c>
+      <c r="N49" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O49" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P49" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q49" s="47" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="48" t="n"/>
+      <c r="B50" s="48" t="n"/>
+      <c r="C50" s="48" t="n"/>
+      <c r="D50" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10005-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E50" s="46" t="inlineStr">
+        <is>
+          <t>Alpha Buffer Left</t>
+        </is>
+      </c>
+      <c r="F50" s="48" t="n"/>
+      <c r="G50" s="48" t="n"/>
+      <c r="H50" s="48" t="n"/>
+      <c r="I50" s="48" t="n"/>
+      <c r="J50" s="48" t="n"/>
+      <c r="K50" s="48" t="n"/>
+      <c r="L50" s="48" t="n"/>
+      <c r="M50" s="48" t="n"/>
+      <c r="N50" s="48" t="n"/>
+      <c r="O50" s="48" t="n"/>
+      <c r="P50" s="48" t="n"/>
+      <c r="Q50" s="48" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="45" t="inlineStr">
+        <is>
+          <t>SB202606091818S07A01</t>
+        </is>
+      </c>
+      <c r="B51" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-F06-60001-X-SUB</t>
+        </is>
+      </c>
+      <c r="C51" s="45" t="inlineStr">
+        <is>
+          <t>Zeta Mount Assembly RH</t>
+        </is>
+      </c>
+      <c r="D51" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-F06-60001-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E51" s="46" t="inlineStr">
+        <is>
+          <t>Zeta Mount RH</t>
+        </is>
+      </c>
+      <c r="F51" s="47" t="inlineStr">
+        <is>
+          <t>WEWW</t>
+        </is>
+      </c>
+      <c r="G51" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H51" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I51" s="47" t="n">
+        <v>130</v>
+      </c>
+      <c r="J51" s="47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K51" s="47" t="inlineStr">
+        <is>
+          <t>543</t>
+        </is>
+      </c>
+      <c r="L51" s="47" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="M51" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09 18:18</t>
+        </is>
+      </c>
+      <c r="N51" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O51" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P51" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q51" s="47" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="48" t="n"/>
+      <c r="B52" s="48" t="n"/>
+      <c r="C52" s="48" t="n"/>
+      <c r="D52" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-F06-60002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E52" s="46" t="inlineStr">
+        <is>
+          <t>Zeta Fastener</t>
+        </is>
+      </c>
+      <c r="F52" s="48" t="n"/>
+      <c r="G52" s="48" t="n"/>
+      <c r="H52" s="48" t="n"/>
+      <c r="I52" s="48" t="n"/>
+      <c r="J52" s="48" t="n"/>
+      <c r="K52" s="48" t="n"/>
+      <c r="L52" s="48" t="n"/>
+      <c r="M52" s="48" t="n"/>
+      <c r="N52" s="48" t="n"/>
+      <c r="O52" s="48" t="n"/>
+      <c r="P52" s="48" t="n"/>
+      <c r="Q52" s="48" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="238">
-    <mergeCell ref="H26:H27"/>
+  <mergeCells count="310">
     <mergeCell ref="N22:N23"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="I30:I33"/>
     <mergeCell ref="P22:P23"/>
-    <mergeCell ref="G8:G9"/>
     <mergeCell ref="K26:K27"/>
     <mergeCell ref="P34:P35"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="O30:O33"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="Q49:Q50"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="H28:H29"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="E44:E46"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="M47:M48"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="J38:J41"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="O4:O5"/>
+    <mergeCell ref="L18:L19"/>
+    <mergeCell ref="F44:F46"/>
+    <mergeCell ref="P36:P37"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="M24:M25"/>
+    <mergeCell ref="C51:C52"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="N30:N33"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="P49:P50"/>
+    <mergeCell ref="M44:M46"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="J26:J27"/>
+    <mergeCell ref="L26:L27"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J18:J19"/>
+    <mergeCell ref="M30:M33"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="I38:I41"/>
+    <mergeCell ref="K38:K41"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="H42:H43"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="P30:P33"/>
+    <mergeCell ref="J42:J43"/>
+    <mergeCell ref="P4:P5"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="K51:K52"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="M51:M52"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="E34:E35"/>
+    <mergeCell ref="G34:G35"/>
+    <mergeCell ref="M10:M13"/>
+    <mergeCell ref="L24:L25"/>
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="I28:I29"/>
+    <mergeCell ref="G10:G13"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="O14:O15"/>
+    <mergeCell ref="O28:O29"/>
+    <mergeCell ref="L44:L46"/>
+    <mergeCell ref="N44:N46"/>
     <mergeCell ref="I16:I17"/>
-    <mergeCell ref="P6:P7"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="A30:A33"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="E38:E41"/>
-    <mergeCell ref="G38:G41"/>
     <mergeCell ref="I26:I27"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="H34:H35"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="O30:O33"/>
     <mergeCell ref="L14:L15"/>
     <mergeCell ref="N14:N15"/>
     <mergeCell ref="I18:I19"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="L30:L33"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="H36:H37"/>
-    <mergeCell ref="J36:J37"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B28:B29"/>
     <mergeCell ref="B38:B41"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="G49:G50"/>
     <mergeCell ref="A22:A23"/>
-    <mergeCell ref="F28:F29"/>
-    <mergeCell ref="I20:I21"/>
-    <mergeCell ref="H28:H29"/>
-    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="H47:H48"/>
+    <mergeCell ref="J47:J48"/>
+    <mergeCell ref="I42:I43"/>
+    <mergeCell ref="K42:K43"/>
+    <mergeCell ref="K44:K46"/>
     <mergeCell ref="J22:J23"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="N24:N25"/>
-    <mergeCell ref="P24:P25"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="P26:P27"/>
+    <mergeCell ref="J51:J52"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="K6:K7"/>
-    <mergeCell ref="L16:L17"/>
-    <mergeCell ref="N16:N17"/>
     <mergeCell ref="F34:F35"/>
-    <mergeCell ref="J38:J41"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="K30:K33"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="G36:G37"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="E14:E15"/>
     <mergeCell ref="F10:F13"/>
-    <mergeCell ref="N26:N27"/>
     <mergeCell ref="M34:M35"/>
-    <mergeCell ref="N18:N19"/>
+    <mergeCell ref="P38:P41"/>
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F36:F37"/>
     <mergeCell ref="H38:H41"/>
-    <mergeCell ref="J34:J35"/>
-    <mergeCell ref="P38:P41"/>
-    <mergeCell ref="O4:O5"/>
-    <mergeCell ref="H10:H13"/>
-    <mergeCell ref="J10:J13"/>
     <mergeCell ref="N2:N3"/>
-    <mergeCell ref="F20:F21"/>
     <mergeCell ref="O36:O37"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="H2:H3"/>
-    <mergeCell ref="L18:L19"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="F22:F23"/>
     <mergeCell ref="J20:J21"/>
-    <mergeCell ref="H22:H23"/>
     <mergeCell ref="L20:L21"/>
-    <mergeCell ref="P36:P37"/>
-    <mergeCell ref="M28:M29"/>
-    <mergeCell ref="O22:O23"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="M24:M25"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="E30:E33"/>
     <mergeCell ref="L22:L23"/>
-    <mergeCell ref="M8:M9"/>
     <mergeCell ref="L34:L35"/>
-    <mergeCell ref="O8:O9"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="B30:B33"/>
     <mergeCell ref="N28:N29"/>
-    <mergeCell ref="N6:N7"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="I34:I35"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="K34:K35"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="K28:K29"/>
-    <mergeCell ref="I10:I13"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="K10:K13"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="H4:H5"/>
     <mergeCell ref="O34:O35"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="O10:O13"/>
     <mergeCell ref="F24:F25"/>
     <mergeCell ref="K20:K21"/>
-    <mergeCell ref="N30:N33"/>
+    <mergeCell ref="M49:M50"/>
     <mergeCell ref="M20:M21"/>
+    <mergeCell ref="O49:O50"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="I47:I48"/>
+    <mergeCell ref="K47:K48"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="L10:L13"/>
+    <mergeCell ref="P28:P29"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="P18:P19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="L36:L37"/>
+    <mergeCell ref="N36:N37"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="M22:M23"/>
+    <mergeCell ref="P16:P17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="J30:J33"/>
+    <mergeCell ref="M36:M37"/>
+    <mergeCell ref="L51:L52"/>
+    <mergeCell ref="N34:N35"/>
+    <mergeCell ref="N10:N13"/>
+    <mergeCell ref="L49:L50"/>
+    <mergeCell ref="N49:N50"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="P42:P43"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="I30:I33"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="P6:P7"/>
+    <mergeCell ref="E38:E41"/>
+    <mergeCell ref="G38:G41"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="L30:L33"/>
+    <mergeCell ref="F42:F43"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="G51:G52"/>
+    <mergeCell ref="I51:I52"/>
+    <mergeCell ref="N24:N25"/>
+    <mergeCell ref="P24:P25"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="P26:P27"/>
+    <mergeCell ref="K30:K33"/>
+    <mergeCell ref="M28:M29"/>
+    <mergeCell ref="H44:H46"/>
+    <mergeCell ref="J44:J46"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="P47:P48"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="C49:C50"/>
     <mergeCell ref="O18:O19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="I36:I37"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="O20:O21"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="J24:J25"/>
-    <mergeCell ref="E28:E29"/>
-    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="E42:E43"/>
+    <mergeCell ref="G42:G43"/>
+    <mergeCell ref="F51:F52"/>
+    <mergeCell ref="H51:H52"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="B34:B35"/>
     <mergeCell ref="G24:G25"/>
     <mergeCell ref="I24:I25"/>
-    <mergeCell ref="A14:A15"/>
     <mergeCell ref="B10:B13"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="L10:L13"/>
-    <mergeCell ref="L26:L27"/>
-    <mergeCell ref="P28:P29"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J18:J19"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="L38:L41"/>
     <mergeCell ref="A4:A5"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="M30:M33"/>
     <mergeCell ref="B36:B37"/>
     <mergeCell ref="F38:F41"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="L38:L41"/>
-    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="H20:H21"/>
+    <mergeCell ref="O38:O41"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="O24:O25"/>
+    <mergeCell ref="J28:J29"/>
+    <mergeCell ref="L28:L29"/>
+    <mergeCell ref="O16:O17"/>
+    <mergeCell ref="G44:G46"/>
+    <mergeCell ref="O26:O27"/>
+    <mergeCell ref="I44:I46"/>
+    <mergeCell ref="Q51:Q52"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="N38:N41"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="M42:M43"/>
+    <mergeCell ref="O42:O43"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="G47:G48"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="N51:N52"/>
+    <mergeCell ref="O6:O7"/>
+    <mergeCell ref="O44:O46"/>
+    <mergeCell ref="P10:P13"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="H34:H35"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="H36:H37"/>
+    <mergeCell ref="J36:J37"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="I20:I21"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="N16:N17"/>
+    <mergeCell ref="F16:F17"/>
+    <mergeCell ref="G36:G37"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="N26:N27"/>
+    <mergeCell ref="P51:P52"/>
+    <mergeCell ref="N18:N19"/>
+    <mergeCell ref="J34:J35"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="J10:J13"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="H49:H50"/>
+    <mergeCell ref="J49:J50"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="L42:L43"/>
+    <mergeCell ref="O47:O48"/>
+    <mergeCell ref="N42:N43"/>
+    <mergeCell ref="O22:O23"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="O51:O52"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="N6:N7"/>
+    <mergeCell ref="I34:I35"/>
+    <mergeCell ref="K34:K35"/>
+    <mergeCell ref="K28:K29"/>
+    <mergeCell ref="I10:I13"/>
+    <mergeCell ref="K10:K13"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I36:I37"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="O20:O21"/>
+    <mergeCell ref="P44:P46"/>
     <mergeCell ref="E16:E17"/>
-    <mergeCell ref="I38:I41"/>
-    <mergeCell ref="K38:K41"/>
     <mergeCell ref="G16:G17"/>
-    <mergeCell ref="P18:P19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="F14:F15"/>
     <mergeCell ref="M26:M27"/>
     <mergeCell ref="P14:P15"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B22:B23"/>
     <mergeCell ref="E18:E19"/>
-    <mergeCell ref="N4:N5"/>
-    <mergeCell ref="H20:H21"/>
-    <mergeCell ref="K16:K17"/>
-    <mergeCell ref="P4:P5"/>
-    <mergeCell ref="P30:P33"/>
-    <mergeCell ref="L36:L37"/>
-    <mergeCell ref="O38:O41"/>
-    <mergeCell ref="N36:N37"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="I49:I50"/>
+    <mergeCell ref="K49:K50"/>
     <mergeCell ref="K36:K37"/>
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="M38:M41"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="O24:O25"/>
-    <mergeCell ref="J28:J29"/>
-    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="L47:L48"/>
+    <mergeCell ref="N47:N48"/>
     <mergeCell ref="M2:M3"/>
-    <mergeCell ref="L28:L29"/>
-    <mergeCell ref="E34:E35"/>
-    <mergeCell ref="O16:O17"/>
-    <mergeCell ref="G34:G35"/>
-    <mergeCell ref="M10:M13"/>
-    <mergeCell ref="L24:L25"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="I28:I29"/>
-    <mergeCell ref="G10:G13"/>
-    <mergeCell ref="K22:K23"/>
-    <mergeCell ref="O26:O27"/>
-    <mergeCell ref="M22:M23"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="N8:N9"/>
     <mergeCell ref="M16:M17"/>
-    <mergeCell ref="P8:P9"/>
     <mergeCell ref="M6:M7"/>
     <mergeCell ref="E6:E7"/>
-    <mergeCell ref="P16:P17"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="J30:J33"/>
-    <mergeCell ref="N38:N41"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="M36:M37"/>
-    <mergeCell ref="K14:K15"/>
     <mergeCell ref="G30:G33"/>
+    <mergeCell ref="A42:A43"/>
     <mergeCell ref="G4:G5"/>
     <mergeCell ref="I4:I5"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="N34:N35"/>
-    <mergeCell ref="N10:N13"/>
-    <mergeCell ref="O14:O15"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="L2:L3"/>
-    <mergeCell ref="M4:M5"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="B51:B52"/>
     <mergeCell ref="N20:N21"/>
     <mergeCell ref="K24:K25"/>
     <mergeCell ref="P20:P21"/>
-    <mergeCell ref="O28:O29"/>
-    <mergeCell ref="O6:O7"/>
     <mergeCell ref="E24:E25"/>
-    <mergeCell ref="P10:P13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3252,221 +4003,405 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="3" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="3" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="3" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" style="27" min="1" max="2"/>
+    <col width="15" customWidth="1" style="27" min="2" max="2"/>
+    <col width="3" customWidth="1" style="27" min="3" max="3"/>
+    <col width="25" customWidth="1" style="27" min="4" max="4"/>
+    <col width="15" customWidth="1" style="27" min="5" max="5"/>
+    <col width="3" customWidth="1" style="27" min="6" max="6"/>
+    <col width="35" customWidth="1" style="27" min="7" max="7"/>
+    <col width="15" customWidth="1" style="27" min="8" max="8"/>
+    <col width="3" customWidth="1" style="27" min="9" max="9"/>
+    <col width="15" customWidth="1" style="27" min="10" max="11"/>
+    <col width="15" customWidth="1" style="27" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="40" t="inlineStr">
-        <is>
-          <t>KPI REPORT | GENERATED: 2026-06-08 19:13 | TOTAL ALL-TIME PRODUCTION: 2218</t>
+      <c r="A1" s="49" t="inlineStr">
+        <is>
+          <t>KPI REPORT | GENERATED: 2026-06-09 18:18 | TOTAL ALL-TIME PRODUCTION: 3602</t>
         </is>
       </c>
     </row>
     <row r="2"/>
-    <row r="4">
-      <c r="A4" s="41" t="inlineStr">
+    <row r="4" ht="20.25" customHeight="1" s="27">
+      <c r="A4" s="50" t="inlineStr">
+        <is>
+          <t>PRODUCTION DATE: 2026-06-09   |   TOTAL DAILY OUTPUT: 1384</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="27">
+      <c r="A5" s="51" t="inlineStr">
+        <is>
+          <t>SHIFT</t>
+        </is>
+      </c>
+      <c r="B5" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="D5" s="51" t="inlineStr">
+        <is>
+          <t>TOP 5 OPERATORS</t>
+        </is>
+      </c>
+      <c r="E5" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="G5" s="51" t="inlineStr">
+        <is>
+          <t>TOP 5 PRODUCTS</t>
+        </is>
+      </c>
+      <c r="H5" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="J5" s="51" t="inlineStr">
+        <is>
+          <t>STATIONS</t>
+        </is>
+      </c>
+      <c r="K5" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" s="27">
+      <c r="A6" s="52" t="inlineStr">
+        <is>
+          <t>Shift A</t>
+        </is>
+      </c>
+      <c r="B6" s="53" t="n">
+        <v>1254</v>
+      </c>
+      <c r="D6" s="52" t="inlineStr">
+        <is>
+          <t>778</t>
+        </is>
+      </c>
+      <c r="E6" s="53" t="n">
+        <v>900</v>
+      </c>
+      <c r="G6" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20001-X-SUB</t>
+        </is>
+      </c>
+      <c r="H6" s="53" t="n">
+        <v>900</v>
+      </c>
+      <c r="J6" s="52" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="K6" s="53" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" s="27">
+      <c r="A7" s="52" t="inlineStr">
+        <is>
+          <t>Shift C</t>
+        </is>
+      </c>
+      <c r="B7" s="53" t="n">
+        <v>130</v>
+      </c>
+      <c r="D7" s="52" t="inlineStr">
+        <is>
+          <t>543</t>
+        </is>
+      </c>
+      <c r="E7" s="53" t="n">
+        <v>260</v>
+      </c>
+      <c r="G7" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-E05-50003-X-SUB</t>
+        </is>
+      </c>
+      <c r="H7" s="53" t="n">
+        <v>134</v>
+      </c>
+      <c r="J7" s="52" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="K7" s="53" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" s="27">
+      <c r="A8" s="52" t="inlineStr"/>
+      <c r="B8" s="52" t="inlineStr"/>
+      <c r="D8" s="52" t="inlineStr">
+        <is>
+          <t>771</t>
+        </is>
+      </c>
+      <c r="E8" s="53" t="n">
+        <v>134</v>
+      </c>
+      <c r="G8" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-F06-60001-X-SUB</t>
+        </is>
+      </c>
+      <c r="H8" s="53" t="n">
+        <v>130</v>
+      </c>
+      <c r="J8" s="52" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="K8" s="53" t="n">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" s="27">
+      <c r="A9" s="52" t="inlineStr"/>
+      <c r="B9" s="52" t="inlineStr"/>
+      <c r="D9" s="52" t="inlineStr">
+        <is>
+          <t>770</t>
+        </is>
+      </c>
+      <c r="E9" s="53" t="n">
+        <v>90</v>
+      </c>
+      <c r="G9" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10006-X-SUB</t>
+        </is>
+      </c>
+      <c r="H9" s="53" t="n">
+        <v>130</v>
+      </c>
+      <c r="J9" s="54" t="inlineStr"/>
+      <c r="K9" s="54" t="inlineStr"/>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" s="27">
+      <c r="A10" s="52" t="inlineStr"/>
+      <c r="B10" s="52" t="inlineStr"/>
+      <c r="D10" s="54" t="inlineStr"/>
+      <c r="E10" s="54" t="inlineStr"/>
+      <c r="G10" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-C03-30006-X-SUB</t>
+        </is>
+      </c>
+      <c r="H10" s="53" t="n">
+        <v>90</v>
+      </c>
+      <c r="J10" s="54" t="inlineStr"/>
+      <c r="K10" s="54" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20.25" customHeight="1" s="27">
+      <c r="A12" s="50" t="inlineStr">
         <is>
           <t>PRODUCTION DATE: 2026-06-08   |   TOTAL DAILY OUTPUT: 2218</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="42" t="inlineStr">
+    <row r="13" ht="16.5" customHeight="1" s="27">
+      <c r="A13" s="51" t="inlineStr">
         <is>
           <t>SHIFT</t>
         </is>
       </c>
-      <c r="B5" s="42" t="inlineStr">
+      <c r="B13" s="51" t="inlineStr">
         <is>
           <t>OUTPUT</t>
         </is>
       </c>
-      <c r="D5" s="42" t="inlineStr">
+      <c r="D13" s="51" t="inlineStr">
         <is>
           <t>TOP 5 OPERATORS</t>
         </is>
       </c>
-      <c r="E5" s="42" t="inlineStr">
+      <c r="E13" s="51" t="inlineStr">
         <is>
           <t>OUTPUT</t>
         </is>
       </c>
-      <c r="G5" s="42" t="inlineStr">
+      <c r="G13" s="51" t="inlineStr">
         <is>
           <t>TOP 5 PRODUCTS</t>
         </is>
       </c>
-      <c r="H5" s="42" t="inlineStr">
+      <c r="H13" s="51" t="inlineStr">
         <is>
           <t>OUTPUT</t>
         </is>
       </c>
-      <c r="J5" s="42" t="inlineStr">
+      <c r="J13" s="51" t="inlineStr">
         <is>
           <t>STATIONS</t>
         </is>
       </c>
-      <c r="K5" s="42" t="inlineStr">
+      <c r="K13" s="51" t="inlineStr">
         <is>
           <t>OUTPUT</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="43" t="inlineStr">
+    <row r="14" ht="16.5" customHeight="1" s="27">
+      <c r="A14" s="52" t="inlineStr">
         <is>
           <t>Shift A</t>
         </is>
       </c>
-      <c r="B6" s="44" t="n">
+      <c r="B14" s="53" t="n">
         <v>1975</v>
       </c>
-      <c r="D6" s="43" t="inlineStr">
+      <c r="D14" s="52" t="inlineStr">
         <is>
           <t>778</t>
         </is>
       </c>
-      <c r="E6" s="44" t="n">
+      <c r="E14" s="53" t="n">
         <v>1164</v>
       </c>
-      <c r="G6" s="43" t="inlineStr">
+      <c r="G14" s="52" t="inlineStr">
         <is>
           <t>MOCK-G07-70001-X-SUB</t>
         </is>
       </c>
-      <c r="H6" s="44" t="n">
+      <c r="H14" s="53" t="n">
         <v>922</v>
       </c>
-      <c r="J6" s="43" t="inlineStr">
+      <c r="J14" s="52" t="inlineStr">
         <is>
           <t>S10</t>
         </is>
       </c>
-      <c r="K6" s="44" t="n">
+      <c r="K14" s="53" t="n">
         <v>1164</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="43" t="inlineStr">
+    <row r="15" ht="16.5" customHeight="1" s="27">
+      <c r="A15" s="52" t="inlineStr">
         <is>
           <t>Shift B</t>
         </is>
       </c>
-      <c r="B7" s="44" t="n">
+      <c r="B15" s="53" t="n">
         <v>243</v>
       </c>
-      <c r="D7" s="43" t="inlineStr">
+      <c r="D15" s="52" t="inlineStr">
         <is>
           <t>777</t>
         </is>
       </c>
-      <c r="E7" s="44" t="n">
+      <c r="E15" s="53" t="n">
         <v>333</v>
       </c>
-      <c r="G7" s="43" t="inlineStr">
+      <c r="G15" s="52" t="inlineStr">
         <is>
           <t>MOCK-A01-10001-X-SUB</t>
         </is>
       </c>
-      <c r="H7" s="44" t="n">
+      <c r="H15" s="53" t="n">
         <v>752</v>
       </c>
-      <c r="J7" s="43" t="inlineStr">
+      <c r="J15" s="52" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
       </c>
-      <c r="K7" s="44" t="n">
+      <c r="K15" s="53" t="n">
         <v>646</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="43" t="inlineStr"/>
-      <c r="B8" s="43" t="inlineStr"/>
-      <c r="D8" s="43" t="inlineStr">
+    <row r="16" ht="16.5" customHeight="1" s="27">
+      <c r="A16" s="52" t="inlineStr"/>
+      <c r="B16" s="52" t="inlineStr"/>
+      <c r="D16" s="52" t="inlineStr">
         <is>
           <t>233</t>
         </is>
       </c>
-      <c r="E8" s="44" t="n">
+      <c r="E16" s="53" t="n">
         <v>234</v>
       </c>
-      <c r="G8" s="43" t="inlineStr">
+      <c r="G16" s="52" t="inlineStr">
         <is>
           <t>MOCK-E05-50003-X-SUB</t>
         </is>
       </c>
-      <c r="H8" s="44" t="n">
+      <c r="H16" s="53" t="n">
         <v>256</v>
       </c>
-      <c r="J8" s="43" t="inlineStr">
+      <c r="J16" s="52" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="K8" s="44" t="n">
+      <c r="K16" s="53" t="n">
         <v>408</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="43" t="inlineStr"/>
-      <c r="B9" s="43" t="inlineStr"/>
-      <c r="D9" s="43" t="inlineStr">
+    <row r="17" ht="16.5" customHeight="1" s="27">
+      <c r="A17" s="52" t="inlineStr"/>
+      <c r="B17" s="52" t="inlineStr"/>
+      <c r="D17" s="52" t="inlineStr">
         <is>
           <t>333</t>
         </is>
       </c>
-      <c r="E9" s="44" t="n">
+      <c r="E17" s="53" t="n">
         <v>123</v>
       </c>
-      <c r="G9" s="43" t="inlineStr">
+      <c r="G17" s="52" t="inlineStr">
         <is>
           <t>MOCK-B02-20004-X-SUB</t>
         </is>
       </c>
-      <c r="H9" s="44" t="n">
+      <c r="H17" s="53" t="n">
         <v>220</v>
       </c>
-      <c r="J9" s="45" t="inlineStr"/>
-      <c r="K9" s="45" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="43" t="inlineStr"/>
-      <c r="B10" s="43" t="inlineStr"/>
-      <c r="D10" s="43" t="inlineStr">
+      <c r="J17" s="54" t="inlineStr"/>
+      <c r="K17" s="54" t="inlineStr"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="27">
+      <c r="A18" s="52" t="inlineStr"/>
+      <c r="B18" s="52" t="inlineStr"/>
+      <c r="D18" s="52" t="inlineStr">
         <is>
           <t>888</t>
         </is>
       </c>
-      <c r="E10" s="44" t="n">
+      <c r="E18" s="53" t="n">
         <v>120</v>
       </c>
-      <c r="G10" s="43" t="inlineStr">
+      <c r="G18" s="52" t="inlineStr">
         <is>
           <t>MOCK-A01-10003-X-SUB</t>
         </is>
       </c>
-      <c r="H10" s="44" t="n">
+      <c r="H18" s="53" t="n">
         <v>68</v>
       </c>
-      <c r="J10" s="45" t="inlineStr"/>
-      <c r="K10" s="45" t="inlineStr"/>
+      <c r="J18" s="54" t="inlineStr"/>
+      <c r="K18" s="54" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A12:K12"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A1:K2"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: implement traceability application logic and build distribution packages
</commit_message>
<xml_diff>
--- a/data/production_data.xlsx
+++ b/data/production_data.xlsx
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q52"/>
+  <dimension ref="A1:Q68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="27" min="1" max="1"/>
@@ -3680,24 +3680,932 @@
       <c r="P52" s="48" t="n"/>
       <c r="Q52" s="48" t="n"/>
     </row>
+    <row r="53">
+      <c r="A53" s="45" t="inlineStr">
+        <is>
+          <t>SB202606101624S06A01</t>
+        </is>
+      </c>
+      <c r="B53" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10001-X-SUB</t>
+        </is>
+      </c>
+      <c r="C53" s="45" t="inlineStr">
+        <is>
+          <t>Alpha Subsystem Right</t>
+        </is>
+      </c>
+      <c r="D53" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10001-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E53" s="46" t="inlineStr">
+        <is>
+          <t>Alpha Core Right</t>
+        </is>
+      </c>
+      <c r="F53" s="47" t="inlineStr">
+        <is>
+          <t>TYTH</t>
+        </is>
+      </c>
+      <c r="G53" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H53" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I53" s="47" t="n">
+        <v>900</v>
+      </c>
+      <c r="J53" s="47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K53" s="47" t="inlineStr">
+        <is>
+          <t>677</t>
+        </is>
+      </c>
+      <c r="L53" s="47" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="M53" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10 16:24</t>
+        </is>
+      </c>
+      <c r="N53" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O53" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P53" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q53" s="47" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="48" t="n"/>
+      <c r="B54" s="48" t="n"/>
+      <c r="C54" s="48" t="n"/>
+      <c r="D54" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E54" s="46" t="inlineStr">
+        <is>
+          <t>Alpha Buffer Right</t>
+        </is>
+      </c>
+      <c r="F54" s="48" t="n"/>
+      <c r="G54" s="48" t="n"/>
+      <c r="H54" s="48" t="n"/>
+      <c r="I54" s="48" t="n"/>
+      <c r="J54" s="48" t="n"/>
+      <c r="K54" s="48" t="n"/>
+      <c r="L54" s="48" t="n"/>
+      <c r="M54" s="48" t="n"/>
+      <c r="N54" s="48" t="n"/>
+      <c r="O54" s="48" t="n"/>
+      <c r="P54" s="48" t="n"/>
+      <c r="Q54" s="48" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="45" t="inlineStr">
+        <is>
+          <t>SB202606101626S06A01</t>
+        </is>
+      </c>
+      <c r="B55" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10003-X-SUB</t>
+        </is>
+      </c>
+      <c r="C55" s="45" t="inlineStr">
+        <is>
+          <t>Alpha Subsystem Aux Right</t>
+        </is>
+      </c>
+      <c r="D55" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10003-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E55" s="46" t="inlineStr">
+        <is>
+          <t>Alpha Core (Auxiliary) Right</t>
+        </is>
+      </c>
+      <c r="F55" s="47" t="inlineStr">
+        <is>
+          <t>HUYL</t>
+        </is>
+      </c>
+      <c r="G55" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H55" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I55" s="47" t="n">
+        <v>890</v>
+      </c>
+      <c r="J55" s="47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K55" s="47" t="inlineStr">
+        <is>
+          <t>666</t>
+        </is>
+      </c>
+      <c r="L55" s="47" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="M55" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10 16:26</t>
+        </is>
+      </c>
+      <c r="N55" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O55" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P55" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q55" s="47" t="inlineStr">
+        <is>
+          <t>999</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="48" t="n"/>
+      <c r="B56" s="48" t="n"/>
+      <c r="C56" s="48" t="n"/>
+      <c r="D56" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E56" s="46" t="inlineStr">
+        <is>
+          <t>Alpha Buffer Right</t>
+        </is>
+      </c>
+      <c r="F56" s="48" t="n"/>
+      <c r="G56" s="48" t="n"/>
+      <c r="H56" s="48" t="n"/>
+      <c r="I56" s="48" t="n"/>
+      <c r="J56" s="48" t="n"/>
+      <c r="K56" s="48" t="n"/>
+      <c r="L56" s="48" t="n"/>
+      <c r="M56" s="48" t="n"/>
+      <c r="N56" s="48" t="n"/>
+      <c r="O56" s="48" t="n"/>
+      <c r="P56" s="48" t="n"/>
+      <c r="Q56" s="48" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="45" t="inlineStr">
+        <is>
+          <t>SB202606101803S07B01</t>
+        </is>
+      </c>
+      <c r="B57" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20005-X-SUB</t>
+        </is>
+      </c>
+      <c r="C57" s="45" t="inlineStr">
+        <is>
+          <t>Beta Panel Left Sub V2</t>
+        </is>
+      </c>
+      <c r="D57" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20005-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E57" s="46" t="inlineStr">
+        <is>
+          <t>Beta Panel (Upgraded) Left</t>
+        </is>
+      </c>
+      <c r="F57" s="47" t="inlineStr">
+        <is>
+          <t>ERRR</t>
+        </is>
+      </c>
+      <c r="G57" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H57" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I57" s="47" t="n">
+        <v>134</v>
+      </c>
+      <c r="J57" s="47" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K57" s="47" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="L57" s="47" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="M57" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10 18:03</t>
+        </is>
+      </c>
+      <c r="N57" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O57" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P57" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q57" s="47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="48" t="n"/>
+      <c r="B58" s="48" t="n"/>
+      <c r="C58" s="48" t="n"/>
+      <c r="D58" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E58" s="46" t="inlineStr">
+        <is>
+          <t>Beta Sealant</t>
+        </is>
+      </c>
+      <c r="F58" s="48" t="n"/>
+      <c r="G58" s="48" t="n"/>
+      <c r="H58" s="48" t="n"/>
+      <c r="I58" s="48" t="n"/>
+      <c r="J58" s="48" t="n"/>
+      <c r="K58" s="48" t="n"/>
+      <c r="L58" s="48" t="n"/>
+      <c r="M58" s="48" t="n"/>
+      <c r="N58" s="48" t="n"/>
+      <c r="O58" s="48" t="n"/>
+      <c r="P58" s="48" t="n"/>
+      <c r="Q58" s="48" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="45" t="inlineStr">
+        <is>
+          <t>SB202606101804S07B01</t>
+        </is>
+      </c>
+      <c r="B59" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20005-X-SUB</t>
+        </is>
+      </c>
+      <c r="C59" s="45" t="inlineStr">
+        <is>
+          <t>Beta Panel Left Sub V2</t>
+        </is>
+      </c>
+      <c r="D59" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20005-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E59" s="46" t="inlineStr">
+        <is>
+          <t>Beta Panel (Upgraded) Left</t>
+        </is>
+      </c>
+      <c r="F59" s="47" t="inlineStr">
+        <is>
+          <t>HHHH</t>
+        </is>
+      </c>
+      <c r="G59" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H59" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I59" s="47" t="n">
+        <v>134</v>
+      </c>
+      <c r="J59" s="47" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K59" s="47" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="L59" s="47" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="M59" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10 18:04</t>
+        </is>
+      </c>
+      <c r="N59" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O59" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P59" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q59" s="47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="48" t="n"/>
+      <c r="B60" s="48" t="n"/>
+      <c r="C60" s="48" t="n"/>
+      <c r="D60" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E60" s="46" t="inlineStr">
+        <is>
+          <t>Beta Sealant</t>
+        </is>
+      </c>
+      <c r="F60" s="48" t="n"/>
+      <c r="G60" s="48" t="n"/>
+      <c r="H60" s="48" t="n"/>
+      <c r="I60" s="48" t="n"/>
+      <c r="J60" s="48" t="n"/>
+      <c r="K60" s="48" t="n"/>
+      <c r="L60" s="48" t="n"/>
+      <c r="M60" s="48" t="n"/>
+      <c r="N60" s="48" t="n"/>
+      <c r="O60" s="48" t="n"/>
+      <c r="P60" s="48" t="n"/>
+      <c r="Q60" s="48" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="45" t="inlineStr">
+        <is>
+          <t>SB202606101811S07A01</t>
+        </is>
+      </c>
+      <c r="B61" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20005-X-SUB</t>
+        </is>
+      </c>
+      <c r="C61" s="45" t="inlineStr">
+        <is>
+          <t>Beta Panel Left Sub V2</t>
+        </is>
+      </c>
+      <c r="D61" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20005-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E61" s="46" t="inlineStr">
+        <is>
+          <t>Beta Panel (Upgraded) Left</t>
+        </is>
+      </c>
+      <c r="F61" s="47" t="inlineStr">
+        <is>
+          <t>UUUU</t>
+        </is>
+      </c>
+      <c r="G61" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H61" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I61" s="47" t="n">
+        <v>134</v>
+      </c>
+      <c r="J61" s="47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K61" s="47" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="L61" s="47" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="M61" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10 18:11</t>
+        </is>
+      </c>
+      <c r="N61" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O61" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P61" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q61" s="47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="48" t="n"/>
+      <c r="B62" s="48" t="n"/>
+      <c r="C62" s="48" t="n"/>
+      <c r="D62" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E62" s="46" t="inlineStr">
+        <is>
+          <t>Beta Sealant</t>
+        </is>
+      </c>
+      <c r="F62" s="48" t="n"/>
+      <c r="G62" s="48" t="n"/>
+      <c r="H62" s="48" t="n"/>
+      <c r="I62" s="48" t="n"/>
+      <c r="J62" s="48" t="n"/>
+      <c r="K62" s="48" t="n"/>
+      <c r="L62" s="48" t="n"/>
+      <c r="M62" s="48" t="n"/>
+      <c r="N62" s="48" t="n"/>
+      <c r="O62" s="48" t="n"/>
+      <c r="P62" s="48" t="n"/>
+      <c r="Q62" s="48" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="45" t="inlineStr">
+        <is>
+          <t>SB202606101812S07A01</t>
+        </is>
+      </c>
+      <c r="B63" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20005-X-SUB</t>
+        </is>
+      </c>
+      <c r="C63" s="45" t="inlineStr">
+        <is>
+          <t>Beta Panel Left Sub V2</t>
+        </is>
+      </c>
+      <c r="D63" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20005-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E63" s="46" t="inlineStr">
+        <is>
+          <t>Beta Panel (Upgraded) Left</t>
+        </is>
+      </c>
+      <c r="F63" s="47" t="inlineStr">
+        <is>
+          <t>YTYTT</t>
+        </is>
+      </c>
+      <c r="G63" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H63" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I63" s="47" t="n">
+        <v>1348</v>
+      </c>
+      <c r="J63" s="47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K63" s="47" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="L63" s="47" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="M63" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10 18:12</t>
+        </is>
+      </c>
+      <c r="N63" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O63" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P63" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q63" s="47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="48" t="n"/>
+      <c r="B64" s="48" t="n"/>
+      <c r="C64" s="48" t="n"/>
+      <c r="D64" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E64" s="46" t="inlineStr">
+        <is>
+          <t>Beta Sealant</t>
+        </is>
+      </c>
+      <c r="F64" s="48" t="n"/>
+      <c r="G64" s="48" t="n"/>
+      <c r="H64" s="48" t="n"/>
+      <c r="I64" s="48" t="n"/>
+      <c r="J64" s="48" t="n"/>
+      <c r="K64" s="48" t="n"/>
+      <c r="L64" s="48" t="n"/>
+      <c r="M64" s="48" t="n"/>
+      <c r="N64" s="48" t="n"/>
+      <c r="O64" s="48" t="n"/>
+      <c r="P64" s="48" t="n"/>
+      <c r="Q64" s="48" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="45" t="inlineStr">
+        <is>
+          <t>SB202606101826S06A01</t>
+        </is>
+      </c>
+      <c r="B65" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-E05-50003-X-SUB</t>
+        </is>
+      </c>
+      <c r="C65" s="45" t="inlineStr">
+        <is>
+          <t>Epsilon Housing Sub Left</t>
+        </is>
+      </c>
+      <c r="D65" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-E05-50003-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E65" s="46" t="inlineStr">
+        <is>
+          <t>Epsilon Housing Left</t>
+        </is>
+      </c>
+      <c r="F65" s="47" t="inlineStr">
+        <is>
+          <t>SDFFGDF</t>
+        </is>
+      </c>
+      <c r="G65" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H65" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I65" s="47" t="n">
+        <v>1400</v>
+      </c>
+      <c r="J65" s="47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K65" s="47" t="inlineStr">
+        <is>
+          <t>5566</t>
+        </is>
+      </c>
+      <c r="L65" s="47" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="M65" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10 18:26</t>
+        </is>
+      </c>
+      <c r="N65" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O65" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P65" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q65" s="47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="48" t="n"/>
+      <c r="B66" s="48" t="n"/>
+      <c r="C66" s="48" t="n"/>
+      <c r="D66" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-E05-50002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E66" s="46" t="inlineStr">
+        <is>
+          <t>Epsilon Axis</t>
+        </is>
+      </c>
+      <c r="F66" s="48" t="n"/>
+      <c r="G66" s="48" t="n"/>
+      <c r="H66" s="48" t="n"/>
+      <c r="I66" s="48" t="n"/>
+      <c r="J66" s="48" t="n"/>
+      <c r="K66" s="48" t="n"/>
+      <c r="L66" s="48" t="n"/>
+      <c r="M66" s="48" t="n"/>
+      <c r="N66" s="48" t="n"/>
+      <c r="O66" s="48" t="n"/>
+      <c r="P66" s="48" t="n"/>
+      <c r="Q66" s="48" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="45" t="inlineStr">
+        <is>
+          <t>SB202606101827S06A01</t>
+        </is>
+      </c>
+      <c r="B67" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10003-X-SUB</t>
+        </is>
+      </c>
+      <c r="C67" s="45" t="inlineStr">
+        <is>
+          <t>Alpha Subsystem Aux Right</t>
+        </is>
+      </c>
+      <c r="D67" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10003-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E67" s="46" t="inlineStr">
+        <is>
+          <t>Alpha Core (Auxiliary) Right</t>
+        </is>
+      </c>
+      <c r="F67" s="47" t="inlineStr">
+        <is>
+          <t>YUYU</t>
+        </is>
+      </c>
+      <c r="G67" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H67" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I67" s="47" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J67" s="47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K67" s="47" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="L67" s="47" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="M67" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10 18:27</t>
+        </is>
+      </c>
+      <c r="N67" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O67" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P67" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q67" s="47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="48" t="n"/>
+      <c r="B68" s="48" t="n"/>
+      <c r="C68" s="48" t="n"/>
+      <c r="D68" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E68" s="46" t="inlineStr">
+        <is>
+          <t>Alpha Buffer Right</t>
+        </is>
+      </c>
+      <c r="F68" s="48" t="n"/>
+      <c r="G68" s="48" t="n"/>
+      <c r="H68" s="48" t="n"/>
+      <c r="I68" s="48" t="n"/>
+      <c r="J68" s="48" t="n"/>
+      <c r="K68" s="48" t="n"/>
+      <c r="L68" s="48" t="n"/>
+      <c r="M68" s="48" t="n"/>
+      <c r="N68" s="48" t="n"/>
+      <c r="O68" s="48" t="n"/>
+      <c r="P68" s="48" t="n"/>
+      <c r="Q68" s="48" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="310">
+  <mergeCells count="430">
     <mergeCell ref="N22:N23"/>
+    <mergeCell ref="K63:K64"/>
     <mergeCell ref="P22:P23"/>
     <mergeCell ref="K26:K27"/>
     <mergeCell ref="P34:P35"/>
     <mergeCell ref="F30:F33"/>
     <mergeCell ref="B42:B43"/>
+    <mergeCell ref="L53:L54"/>
+    <mergeCell ref="N53:N54"/>
+    <mergeCell ref="I57:I58"/>
     <mergeCell ref="O30:O33"/>
+    <mergeCell ref="J55:J56"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="L55:L56"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="Q49:Q50"/>
     <mergeCell ref="F28:F29"/>
     <mergeCell ref="H28:H29"/>
     <mergeCell ref="M18:M19"/>
+    <mergeCell ref="O67:O68"/>
     <mergeCell ref="E44:E46"/>
+    <mergeCell ref="K53:K54"/>
+    <mergeCell ref="F57:F58"/>
     <mergeCell ref="H8:H9"/>
+    <mergeCell ref="M53:M54"/>
     <mergeCell ref="M47:M48"/>
     <mergeCell ref="J8:J9"/>
+    <mergeCell ref="K55:K56"/>
     <mergeCell ref="B26:B27"/>
     <mergeCell ref="J38:J41"/>
     <mergeCell ref="E14:E15"/>
@@ -3708,11 +4616,18 @@
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="M24:M25"/>
     <mergeCell ref="C51:C52"/>
+    <mergeCell ref="A63:A64"/>
+    <mergeCell ref="O57:O58"/>
+    <mergeCell ref="Q57:Q58"/>
     <mergeCell ref="A38:A41"/>
     <mergeCell ref="N30:N33"/>
+    <mergeCell ref="F65:F66"/>
     <mergeCell ref="E20:E21"/>
+    <mergeCell ref="M55:M56"/>
     <mergeCell ref="A6:A7"/>
+    <mergeCell ref="K59:K60"/>
     <mergeCell ref="P49:P50"/>
+    <mergeCell ref="C59:C60"/>
     <mergeCell ref="M44:M46"/>
     <mergeCell ref="J24:J25"/>
     <mergeCell ref="E28:E29"/>
@@ -3749,12 +4664,21 @@
     <mergeCell ref="I28:I29"/>
     <mergeCell ref="G10:G13"/>
     <mergeCell ref="A18:A19"/>
+    <mergeCell ref="N57:N58"/>
+    <mergeCell ref="K67:K68"/>
+    <mergeCell ref="P57:P58"/>
+    <mergeCell ref="C67:C68"/>
+    <mergeCell ref="C61:C62"/>
+    <mergeCell ref="L65:L66"/>
     <mergeCell ref="E36:E37"/>
     <mergeCell ref="A47:A48"/>
+    <mergeCell ref="N65:N66"/>
     <mergeCell ref="O14:O15"/>
     <mergeCell ref="O28:O29"/>
+    <mergeCell ref="B59:B60"/>
     <mergeCell ref="L44:L46"/>
     <mergeCell ref="N44:N46"/>
+    <mergeCell ref="B61:B62"/>
     <mergeCell ref="I16:I17"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="A30:A33"/>
@@ -3764,6 +4688,7 @@
     <mergeCell ref="I18:I19"/>
     <mergeCell ref="B38:B41"/>
     <mergeCell ref="G49:G50"/>
+    <mergeCell ref="C57:C58"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="H47:H48"/>
     <mergeCell ref="J47:J48"/>
@@ -3771,10 +4696,14 @@
     <mergeCell ref="K42:K43"/>
     <mergeCell ref="K44:K46"/>
     <mergeCell ref="J22:J23"/>
+    <mergeCell ref="A53:A54"/>
     <mergeCell ref="J51:J52"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="K6:K7"/>
+    <mergeCell ref="F63:F64"/>
     <mergeCell ref="F34:F35"/>
+    <mergeCell ref="M59:M60"/>
+    <mergeCell ref="H63:H64"/>
     <mergeCell ref="F10:F13"/>
     <mergeCell ref="M34:M35"/>
     <mergeCell ref="P38:P41"/>
@@ -3786,8 +4715,12 @@
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="H2:H3"/>
+    <mergeCell ref="B67:B68"/>
+    <mergeCell ref="M65:M66"/>
     <mergeCell ref="J20:J21"/>
+    <mergeCell ref="O65:O66"/>
     <mergeCell ref="L20:L21"/>
+    <mergeCell ref="G63:G64"/>
     <mergeCell ref="L22:L23"/>
     <mergeCell ref="L34:L35"/>
     <mergeCell ref="B30:B33"/>
@@ -3802,22 +4735,35 @@
     <mergeCell ref="O49:O50"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="A44:A46"/>
+    <mergeCell ref="G53:G54"/>
+    <mergeCell ref="B57:B58"/>
+    <mergeCell ref="I53:I54"/>
     <mergeCell ref="F8:F9"/>
     <mergeCell ref="I47:I48"/>
     <mergeCell ref="K47:K48"/>
+    <mergeCell ref="O55:O56"/>
+    <mergeCell ref="G55:G56"/>
     <mergeCell ref="A14:A15"/>
     <mergeCell ref="L10:L13"/>
     <mergeCell ref="P28:P29"/>
     <mergeCell ref="H16:H17"/>
     <mergeCell ref="K4:K5"/>
+    <mergeCell ref="L59:L60"/>
+    <mergeCell ref="N59:N60"/>
     <mergeCell ref="P18:P19"/>
+    <mergeCell ref="I63:I64"/>
     <mergeCell ref="H18:H19"/>
+    <mergeCell ref="H67:H68"/>
+    <mergeCell ref="J67:J68"/>
     <mergeCell ref="B4:B5"/>
+    <mergeCell ref="J61:J62"/>
+    <mergeCell ref="L61:L62"/>
     <mergeCell ref="B44:B46"/>
     <mergeCell ref="K16:K17"/>
     <mergeCell ref="L36:L37"/>
     <mergeCell ref="N36:N37"/>
     <mergeCell ref="G2:G3"/>
+    <mergeCell ref="A67:A68"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="I22:I23"/>
     <mergeCell ref="K22:K23"/>
@@ -3826,42 +4772,69 @@
     <mergeCell ref="J16:J17"/>
     <mergeCell ref="J30:J33"/>
     <mergeCell ref="M36:M37"/>
+    <mergeCell ref="B65:B66"/>
     <mergeCell ref="L51:L52"/>
+    <mergeCell ref="I55:I56"/>
     <mergeCell ref="N34:N35"/>
     <mergeCell ref="N10:N13"/>
+    <mergeCell ref="G59:G60"/>
     <mergeCell ref="L49:L50"/>
+    <mergeCell ref="I59:I60"/>
     <mergeCell ref="N49:N50"/>
     <mergeCell ref="M4:M5"/>
     <mergeCell ref="A34:A35"/>
     <mergeCell ref="A28:A29"/>
     <mergeCell ref="P42:P43"/>
+    <mergeCell ref="L67:L68"/>
+    <mergeCell ref="F53:F54"/>
     <mergeCell ref="H26:H27"/>
+    <mergeCell ref="H53:H54"/>
     <mergeCell ref="E8:E9"/>
     <mergeCell ref="I30:I33"/>
     <mergeCell ref="G8:G9"/>
     <mergeCell ref="P6:P7"/>
     <mergeCell ref="E38:E41"/>
+    <mergeCell ref="F55:F56"/>
     <mergeCell ref="G38:G41"/>
+    <mergeCell ref="H55:H56"/>
     <mergeCell ref="B14:B15"/>
+    <mergeCell ref="O63:O64"/>
+    <mergeCell ref="Q63:Q64"/>
     <mergeCell ref="J4:J5"/>
     <mergeCell ref="L30:L33"/>
     <mergeCell ref="F42:F43"/>
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="G18:G19"/>
+    <mergeCell ref="I67:I68"/>
+    <mergeCell ref="K61:K62"/>
     <mergeCell ref="G51:G52"/>
+    <mergeCell ref="M61:M62"/>
     <mergeCell ref="I51:I52"/>
     <mergeCell ref="N24:N25"/>
     <mergeCell ref="P24:P25"/>
     <mergeCell ref="H24:H25"/>
     <mergeCell ref="A10:A13"/>
     <mergeCell ref="P26:P27"/>
+    <mergeCell ref="A59:A60"/>
     <mergeCell ref="K30:K33"/>
+    <mergeCell ref="O53:O54"/>
+    <mergeCell ref="J57:J58"/>
+    <mergeCell ref="Q53:Q54"/>
+    <mergeCell ref="L57:L58"/>
+    <mergeCell ref="A61:A62"/>
+    <mergeCell ref="Q55:Q56"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="C65:C66"/>
     <mergeCell ref="M28:M29"/>
     <mergeCell ref="H44:H46"/>
     <mergeCell ref="J44:J46"/>
+    <mergeCell ref="P53:P54"/>
+    <mergeCell ref="K57:K58"/>
+    <mergeCell ref="F61:F62"/>
     <mergeCell ref="M8:M9"/>
     <mergeCell ref="P47:P48"/>
+    <mergeCell ref="M57:M58"/>
     <mergeCell ref="O8:O9"/>
     <mergeCell ref="O2:O3"/>
     <mergeCell ref="E26:E27"/>
@@ -3870,9 +4843,12 @@
     <mergeCell ref="J14:J15"/>
     <mergeCell ref="A49:A50"/>
     <mergeCell ref="C49:C50"/>
+    <mergeCell ref="N63:N64"/>
+    <mergeCell ref="P63:P64"/>
     <mergeCell ref="O18:O19"/>
     <mergeCell ref="E42:E43"/>
     <mergeCell ref="G42:G43"/>
+    <mergeCell ref="J65:J66"/>
     <mergeCell ref="F51:F52"/>
     <mergeCell ref="H51:H52"/>
     <mergeCell ref="G6:G7"/>
@@ -3884,14 +4860,20 @@
     <mergeCell ref="L38:L41"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="B36:B37"/>
+    <mergeCell ref="Q61:Q62"/>
     <mergeCell ref="F38:F41"/>
+    <mergeCell ref="I65:I66"/>
+    <mergeCell ref="K65:K66"/>
+    <mergeCell ref="N55:N56"/>
     <mergeCell ref="H20:H21"/>
     <mergeCell ref="O38:O41"/>
+    <mergeCell ref="P55:P56"/>
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="O24:O25"/>
     <mergeCell ref="J28:J29"/>
     <mergeCell ref="L28:L29"/>
     <mergeCell ref="O16:O17"/>
+    <mergeCell ref="Q67:Q68"/>
     <mergeCell ref="G44:G46"/>
     <mergeCell ref="O26:O27"/>
     <mergeCell ref="I44:I46"/>
@@ -3907,6 +4889,7 @@
     <mergeCell ref="K14:K15"/>
     <mergeCell ref="M42:M43"/>
     <mergeCell ref="O42:O43"/>
+    <mergeCell ref="C53:C54"/>
     <mergeCell ref="E47:E48"/>
     <mergeCell ref="G47:G48"/>
     <mergeCell ref="E22:E23"/>
@@ -3915,16 +4898,28 @@
     <mergeCell ref="O44:O46"/>
     <mergeCell ref="P10:P13"/>
     <mergeCell ref="A51:A52"/>
+    <mergeCell ref="F59:F60"/>
+    <mergeCell ref="P59:P60"/>
+    <mergeCell ref="C63:C64"/>
+    <mergeCell ref="H59:H60"/>
+    <mergeCell ref="J59:J60"/>
     <mergeCell ref="H34:H35"/>
     <mergeCell ref="F18:F19"/>
+    <mergeCell ref="N67:N68"/>
+    <mergeCell ref="N61:N62"/>
+    <mergeCell ref="P67:P68"/>
+    <mergeCell ref="P61:P62"/>
+    <mergeCell ref="H61:H62"/>
     <mergeCell ref="F26:F27"/>
     <mergeCell ref="H36:H37"/>
     <mergeCell ref="J36:J37"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="F47:F48"/>
     <mergeCell ref="E2:E3"/>
+    <mergeCell ref="H65:H66"/>
     <mergeCell ref="I20:I21"/>
     <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B63:B64"/>
     <mergeCell ref="G22:G23"/>
     <mergeCell ref="L16:L17"/>
     <mergeCell ref="N16:N17"/>
@@ -3947,23 +4942,34 @@
     <mergeCell ref="O47:O48"/>
     <mergeCell ref="N42:N43"/>
     <mergeCell ref="O22:O23"/>
+    <mergeCell ref="B53:B54"/>
+    <mergeCell ref="Q65:Q66"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="E30:E33"/>
+    <mergeCell ref="A57:A58"/>
     <mergeCell ref="O51:O52"/>
     <mergeCell ref="L6:L7"/>
+    <mergeCell ref="B55:B56"/>
     <mergeCell ref="N6:N7"/>
     <mergeCell ref="I34:I35"/>
     <mergeCell ref="K34:K35"/>
+    <mergeCell ref="M63:M64"/>
     <mergeCell ref="K28:K29"/>
     <mergeCell ref="I10:I13"/>
     <mergeCell ref="K10:K13"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="H4:H5"/>
+    <mergeCell ref="M67:M68"/>
+    <mergeCell ref="G67:G68"/>
+    <mergeCell ref="G61:G62"/>
+    <mergeCell ref="I61:I62"/>
+    <mergeCell ref="P65:P66"/>
     <mergeCell ref="I36:I37"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="A36:A37"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="O20:O21"/>
+    <mergeCell ref="H57:H58"/>
     <mergeCell ref="P44:P46"/>
     <mergeCell ref="E16:E17"/>
     <mergeCell ref="G16:G17"/>
@@ -3975,18 +4981,28 @@
     <mergeCell ref="K36:K37"/>
     <mergeCell ref="A24:A25"/>
     <mergeCell ref="M38:M41"/>
+    <mergeCell ref="J53:J54"/>
+    <mergeCell ref="G57:G58"/>
     <mergeCell ref="L47:L48"/>
     <mergeCell ref="N47:N48"/>
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="M16:M17"/>
+    <mergeCell ref="A55:A56"/>
     <mergeCell ref="M6:M7"/>
+    <mergeCell ref="C55:C56"/>
     <mergeCell ref="E6:E7"/>
+    <mergeCell ref="O59:O60"/>
+    <mergeCell ref="J63:J64"/>
+    <mergeCell ref="Q59:Q60"/>
+    <mergeCell ref="L63:L64"/>
     <mergeCell ref="G30:G33"/>
     <mergeCell ref="A42:A43"/>
     <mergeCell ref="G4:G5"/>
+    <mergeCell ref="O61:O62"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="L2:L3"/>
+    <mergeCell ref="F67:F68"/>
     <mergeCell ref="B51:B52"/>
     <mergeCell ref="N20:N21"/>
     <mergeCell ref="K24:K25"/>
@@ -4003,7 +5019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" style="27" min="1" max="2"/>
@@ -4022,7 +5038,7 @@
     <row r="1">
       <c r="A1" s="49" t="inlineStr">
         <is>
-          <t>KPI REPORT | GENERATED: 2026-06-09 18:18 | TOTAL ALL-TIME PRODUCTION: 3602</t>
+          <t>KPI REPORT | GENERATED: 2026-06-10 18:27 | TOTAL ALL-TIME PRODUCTION: 13542</t>
         </is>
       </c>
     </row>
@@ -4030,7 +5046,7 @@
     <row r="4" ht="20.25" customHeight="1" s="27">
       <c r="A4" s="50" t="inlineStr">
         <is>
-          <t>PRODUCTION DATE: 2026-06-09   |   TOTAL DAILY OUTPUT: 1384</t>
+          <t>PRODUCTION DATE: 2026-06-10   |   TOTAL DAILY OUTPUT: 9940</t>
         </is>
       </c>
     </row>
@@ -4083,57 +5099,57 @@
         </is>
       </c>
       <c r="B6" s="53" t="n">
-        <v>1254</v>
+        <v>9672</v>
       </c>
       <c r="D6" s="52" t="inlineStr">
         <is>
-          <t>778</t>
+          <t>111</t>
         </is>
       </c>
       <c r="E6" s="53" t="n">
-        <v>900</v>
+        <v>5000</v>
       </c>
       <c r="G6" s="52" t="inlineStr">
         <is>
-          <t>MOCK-B02-20001-X-SUB</t>
+          <t>MOCK-A01-10003-X-SUB</t>
         </is>
       </c>
       <c r="H6" s="53" t="n">
-        <v>900</v>
+        <v>5890</v>
       </c>
       <c r="J6" s="52" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S06</t>
         </is>
       </c>
       <c r="K6" s="53" t="n">
-        <v>900</v>
+        <v>8190</v>
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1" s="27">
       <c r="A7" s="52" t="inlineStr">
         <is>
-          <t>Shift C</t>
+          <t>Shift B</t>
         </is>
       </c>
       <c r="B7" s="53" t="n">
-        <v>130</v>
+        <v>268</v>
       </c>
       <c r="D7" s="52" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>333</t>
         </is>
       </c>
       <c r="E7" s="53" t="n">
-        <v>260</v>
+        <v>1750</v>
       </c>
       <c r="G7" s="52" t="inlineStr">
         <is>
-          <t>MOCK-E05-50003-X-SUB</t>
+          <t>MOCK-B02-20005-X-SUB</t>
         </is>
       </c>
       <c r="H7" s="53" t="n">
-        <v>134</v>
+        <v>1750</v>
       </c>
       <c r="J7" s="52" t="inlineStr">
         <is>
@@ -4141,7 +5157,7 @@
         </is>
       </c>
       <c r="K7" s="53" t="n">
-        <v>260</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="8" ht="16.5" customHeight="1" s="27">
@@ -4149,47 +5165,41 @@
       <c r="B8" s="52" t="inlineStr"/>
       <c r="D8" s="52" t="inlineStr">
         <is>
-          <t>771</t>
+          <t>5566</t>
         </is>
       </c>
       <c r="E8" s="53" t="n">
-        <v>134</v>
+        <v>1400</v>
       </c>
       <c r="G8" s="52" t="inlineStr">
         <is>
-          <t>MOCK-F06-60001-X-SUB</t>
+          <t>MOCK-E05-50003-X-SUB</t>
         </is>
       </c>
       <c r="H8" s="53" t="n">
-        <v>130</v>
-      </c>
-      <c r="J8" s="52" t="inlineStr">
-        <is>
-          <t>S11</t>
-        </is>
-      </c>
-      <c r="K8" s="53" t="n">
-        <v>224</v>
-      </c>
+        <v>1400</v>
+      </c>
+      <c r="J8" s="54" t="inlineStr"/>
+      <c r="K8" s="54" t="inlineStr"/>
     </row>
     <row r="9" ht="16.5" customHeight="1" s="27">
       <c r="A9" s="52" t="inlineStr"/>
       <c r="B9" s="52" t="inlineStr"/>
       <c r="D9" s="52" t="inlineStr">
         <is>
-          <t>770</t>
+          <t>677</t>
         </is>
       </c>
       <c r="E9" s="53" t="n">
-        <v>90</v>
+        <v>900</v>
       </c>
       <c r="G9" s="52" t="inlineStr">
         <is>
-          <t>MOCK-A01-10006-X-SUB</t>
+          <t>MOCK-A01-10001-X-SUB</t>
         </is>
       </c>
       <c r="H9" s="53" t="n">
-        <v>130</v>
+        <v>900</v>
       </c>
       <c r="J9" s="54" t="inlineStr"/>
       <c r="K9" s="54" t="inlineStr"/>
@@ -4197,23 +5207,23 @@
     <row r="10" ht="16.5" customHeight="1" s="27">
       <c r="A10" s="52" t="inlineStr"/>
       <c r="B10" s="52" t="inlineStr"/>
-      <c r="D10" s="54" t="inlineStr"/>
-      <c r="E10" s="54" t="inlineStr"/>
-      <c r="G10" s="52" t="inlineStr">
-        <is>
-          <t>MOCK-C03-30006-X-SUB</t>
-        </is>
-      </c>
-      <c r="H10" s="53" t="n">
-        <v>90</v>
-      </c>
+      <c r="D10" s="52" t="inlineStr">
+        <is>
+          <t>666</t>
+        </is>
+      </c>
+      <c r="E10" s="53" t="n">
+        <v>890</v>
+      </c>
+      <c r="G10" s="54" t="inlineStr"/>
+      <c r="H10" s="54" t="inlineStr"/>
       <c r="J10" s="54" t="inlineStr"/>
       <c r="K10" s="54" t="inlineStr"/>
     </row>
     <row r="12" ht="20.25" customHeight="1" s="27">
       <c r="A12" s="50" t="inlineStr">
         <is>
-          <t>PRODUCTION DATE: 2026-06-08   |   TOTAL DAILY OUTPUT: 2218</t>
+          <t>PRODUCTION DATE: 2026-06-09   |   TOTAL DAILY OUTPUT: 1384</t>
         </is>
       </c>
     </row>
@@ -4266,7 +5276,7 @@
         </is>
       </c>
       <c r="B14" s="53" t="n">
-        <v>1975</v>
+        <v>1254</v>
       </c>
       <c r="D14" s="52" t="inlineStr">
         <is>
@@ -4274,15 +5284,15 @@
         </is>
       </c>
       <c r="E14" s="53" t="n">
-        <v>1164</v>
+        <v>900</v>
       </c>
       <c r="G14" s="52" t="inlineStr">
         <is>
-          <t>MOCK-G07-70001-X-SUB</t>
+          <t>MOCK-B02-20001-X-SUB</t>
         </is>
       </c>
       <c r="H14" s="53" t="n">
-        <v>922</v>
+        <v>900</v>
       </c>
       <c r="J14" s="52" t="inlineStr">
         <is>
@@ -4290,33 +5300,33 @@
         </is>
       </c>
       <c r="K14" s="53" t="n">
-        <v>1164</v>
+        <v>900</v>
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1" s="27">
       <c r="A15" s="52" t="inlineStr">
         <is>
-          <t>Shift B</t>
+          <t>Shift C</t>
         </is>
       </c>
       <c r="B15" s="53" t="n">
-        <v>243</v>
+        <v>130</v>
       </c>
       <c r="D15" s="52" t="inlineStr">
         <is>
-          <t>777</t>
+          <t>543</t>
         </is>
       </c>
       <c r="E15" s="53" t="n">
-        <v>333</v>
+        <v>260</v>
       </c>
       <c r="G15" s="52" t="inlineStr">
         <is>
-          <t>MOCK-A01-10001-X-SUB</t>
+          <t>MOCK-E05-50003-X-SUB</t>
         </is>
       </c>
       <c r="H15" s="53" t="n">
-        <v>752</v>
+        <v>134</v>
       </c>
       <c r="J15" s="52" t="inlineStr">
         <is>
@@ -4324,7 +5334,7 @@
         </is>
       </c>
       <c r="K15" s="53" t="n">
-        <v>646</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="27">
@@ -4332,27 +5342,27 @@
       <c r="B16" s="52" t="inlineStr"/>
       <c r="D16" s="52" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>771</t>
         </is>
       </c>
       <c r="E16" s="53" t="n">
-        <v>234</v>
+        <v>134</v>
       </c>
       <c r="G16" s="52" t="inlineStr">
         <is>
-          <t>MOCK-E05-50003-X-SUB</t>
+          <t>MOCK-A01-10006-X-SUB</t>
         </is>
       </c>
       <c r="H16" s="53" t="n">
-        <v>256</v>
+        <v>130</v>
       </c>
       <c r="J16" s="52" t="inlineStr">
         <is>
-          <t>S06</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="K16" s="53" t="n">
-        <v>408</v>
+        <v>224</v>
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1" s="27">
@@ -4360,19 +5370,19 @@
       <c r="B17" s="52" t="inlineStr"/>
       <c r="D17" s="52" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>770</t>
         </is>
       </c>
       <c r="E17" s="53" t="n">
-        <v>123</v>
+        <v>90</v>
       </c>
       <c r="G17" s="52" t="inlineStr">
         <is>
-          <t>MOCK-B02-20004-X-SUB</t>
+          <t>MOCK-F06-60001-X-SUB</t>
         </is>
       </c>
       <c r="H17" s="53" t="n">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="J17" s="54" t="inlineStr"/>
       <c r="K17" s="54" t="inlineStr"/>
@@ -4380,30 +5390,214 @@
     <row r="18" ht="16.5" customHeight="1" s="27">
       <c r="A18" s="52" t="inlineStr"/>
       <c r="B18" s="52" t="inlineStr"/>
-      <c r="D18" s="52" t="inlineStr">
-        <is>
-          <t>888</t>
-        </is>
-      </c>
-      <c r="E18" s="53" t="n">
-        <v>120</v>
-      </c>
+      <c r="D18" s="54" t="inlineStr"/>
+      <c r="E18" s="54" t="inlineStr"/>
       <c r="G18" s="52" t="inlineStr">
         <is>
-          <t>MOCK-A01-10003-X-SUB</t>
+          <t>MOCK-C03-30006-X-SUB</t>
         </is>
       </c>
       <c r="H18" s="53" t="n">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="J18" s="54" t="inlineStr"/>
       <c r="K18" s="54" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="50" t="inlineStr">
+        <is>
+          <t>PRODUCTION DATE: 2026-06-08   |   TOTAL DAILY OUTPUT: 2218</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="51" t="inlineStr">
+        <is>
+          <t>SHIFT</t>
+        </is>
+      </c>
+      <c r="B21" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="D21" s="51" t="inlineStr">
+        <is>
+          <t>TOP 5 OPERATORS</t>
+        </is>
+      </c>
+      <c r="E21" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="G21" s="51" t="inlineStr">
+        <is>
+          <t>TOP 5 PRODUCTS</t>
+        </is>
+      </c>
+      <c r="H21" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="J21" s="51" t="inlineStr">
+        <is>
+          <t>STATIONS</t>
+        </is>
+      </c>
+      <c r="K21" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="52" t="inlineStr">
+        <is>
+          <t>Shift A</t>
+        </is>
+      </c>
+      <c r="B22" s="53" t="n">
+        <v>1975</v>
+      </c>
+      <c r="D22" s="52" t="inlineStr">
+        <is>
+          <t>778</t>
+        </is>
+      </c>
+      <c r="E22" s="53" t="n">
+        <v>1164</v>
+      </c>
+      <c r="G22" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-G07-70001-X-SUB</t>
+        </is>
+      </c>
+      <c r="H22" s="53" t="n">
+        <v>922</v>
+      </c>
+      <c r="J22" s="52" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="K22" s="53" t="n">
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="52" t="inlineStr">
+        <is>
+          <t>Shift B</t>
+        </is>
+      </c>
+      <c r="B23" s="53" t="n">
+        <v>243</v>
+      </c>
+      <c r="D23" s="52" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E23" s="53" t="n">
+        <v>333</v>
+      </c>
+      <c r="G23" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10001-X-SUB</t>
+        </is>
+      </c>
+      <c r="H23" s="53" t="n">
+        <v>752</v>
+      </c>
+      <c r="J23" s="52" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="K23" s="53" t="n">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="52" t="inlineStr"/>
+      <c r="B24" s="52" t="inlineStr"/>
+      <c r="D24" s="52" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="E24" s="53" t="n">
+        <v>234</v>
+      </c>
+      <c r="G24" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-E05-50003-X-SUB</t>
+        </is>
+      </c>
+      <c r="H24" s="53" t="n">
+        <v>256</v>
+      </c>
+      <c r="J24" s="52" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="K24" s="53" t="n">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="52" t="inlineStr"/>
+      <c r="B25" s="52" t="inlineStr"/>
+      <c r="D25" s="52" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="E25" s="53" t="n">
+        <v>123</v>
+      </c>
+      <c r="G25" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20004-X-SUB</t>
+        </is>
+      </c>
+      <c r="H25" s="53" t="n">
+        <v>220</v>
+      </c>
+      <c r="J25" s="54" t="inlineStr"/>
+      <c r="K25" s="54" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="52" t="inlineStr"/>
+      <c r="B26" s="52" t="inlineStr"/>
+      <c r="D26" s="52" t="inlineStr">
+        <is>
+          <t>888</t>
+        </is>
+      </c>
+      <c r="E26" s="53" t="n">
+        <v>120</v>
+      </c>
+      <c r="G26" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10003-X-SUB</t>
+        </is>
+      </c>
+      <c r="H26" s="53" t="n">
+        <v>68</v>
+      </c>
+      <c r="J26" s="54" t="inlineStr"/>
+      <c r="K26" s="54" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="A1:K2"/>
     <mergeCell ref="A12:K12"/>
     <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A1:K2"/>
+    <mergeCell ref="A20:K20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: generate traceability reports, ZPL labels, and application build artifacts
</commit_message>
<xml_diff>
--- a/data/production_data.xlsx
+++ b/data/production_data.xlsx
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q68"/>
+  <dimension ref="A1:Q72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="27" min="1" max="1"/>
@@ -4576,8 +4576,232 @@
       <c r="P68" s="48" t="n"/>
       <c r="Q68" s="48" t="n"/>
     </row>
+    <row r="69">
+      <c r="A69" s="45" t="inlineStr">
+        <is>
+          <t>SB202606112038S06A01</t>
+        </is>
+      </c>
+      <c r="B69" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10003-X-SUB</t>
+        </is>
+      </c>
+      <c r="C69" s="45" t="inlineStr">
+        <is>
+          <t>Alpha Subsystem Aux Right</t>
+        </is>
+      </c>
+      <c r="D69" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10003-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E69" s="46" t="inlineStr">
+        <is>
+          <t>Alpha Core (Auxiliary) Right</t>
+        </is>
+      </c>
+      <c r="F69" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G69" s="47" t="inlineStr">
+        <is>
+          <t>HUIK</t>
+        </is>
+      </c>
+      <c r="H69" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I69" s="47" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J69" s="47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K69" s="47" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="L69" s="47" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="M69" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-11 20:38</t>
+        </is>
+      </c>
+      <c r="N69" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O69" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P69" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q69" s="47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="48" t="n"/>
+      <c r="B70" s="48" t="n"/>
+      <c r="C70" s="48" t="n"/>
+      <c r="D70" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E70" s="46" t="inlineStr">
+        <is>
+          <t>Alpha Buffer Right</t>
+        </is>
+      </c>
+      <c r="F70" s="48" t="n"/>
+      <c r="G70" s="48" t="n"/>
+      <c r="H70" s="48" t="n"/>
+      <c r="I70" s="48" t="n"/>
+      <c r="J70" s="48" t="n"/>
+      <c r="K70" s="48" t="n"/>
+      <c r="L70" s="48" t="n"/>
+      <c r="M70" s="48" t="n"/>
+      <c r="N70" s="48" t="n"/>
+      <c r="O70" s="48" t="n"/>
+      <c r="P70" s="48" t="n"/>
+      <c r="Q70" s="48" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="45" t="inlineStr">
+        <is>
+          <t>SB202606112044S06A01</t>
+        </is>
+      </c>
+      <c r="B71" s="45" t="inlineStr">
+        <is>
+          <t>MOCK-F06-60001-X-SUB</t>
+        </is>
+      </c>
+      <c r="C71" s="45" t="inlineStr">
+        <is>
+          <t>Zeta Mount Assembly RH</t>
+        </is>
+      </c>
+      <c r="D71" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-F06-60001-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E71" s="46" t="inlineStr">
+        <is>
+          <t>Zeta Mount RH</t>
+        </is>
+      </c>
+      <c r="F71" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G71" s="47" t="inlineStr">
+        <is>
+          <t>IO0K</t>
+        </is>
+      </c>
+      <c r="H71" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I71" s="47" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J71" s="47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K71" s="47" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="L71" s="47" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="M71" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-11 20:44</t>
+        </is>
+      </c>
+      <c r="N71" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O71" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P71" s="47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q71" s="47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="48" t="n"/>
+      <c r="B72" s="48" t="n"/>
+      <c r="C72" s="48" t="n"/>
+      <c r="D72" s="46" t="inlineStr">
+        <is>
+          <t>MOCK-F06-60002-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E72" s="46" t="inlineStr">
+        <is>
+          <t>Zeta Fastener</t>
+        </is>
+      </c>
+      <c r="F72" s="48" t="n"/>
+      <c r="G72" s="48" t="n"/>
+      <c r="H72" s="48" t="n"/>
+      <c r="I72" s="48" t="n"/>
+      <c r="J72" s="48" t="n"/>
+      <c r="K72" s="48" t="n"/>
+      <c r="L72" s="48" t="n"/>
+      <c r="M72" s="48" t="n"/>
+      <c r="N72" s="48" t="n"/>
+      <c r="O72" s="48" t="n"/>
+      <c r="P72" s="48" t="n"/>
+      <c r="Q72" s="48" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="430">
+  <mergeCells count="460">
     <mergeCell ref="N22:N23"/>
     <mergeCell ref="K63:K64"/>
     <mergeCell ref="P22:P23"/>
@@ -4598,6 +4822,7 @@
     <mergeCell ref="H28:H29"/>
     <mergeCell ref="M18:M19"/>
     <mergeCell ref="O67:O68"/>
+    <mergeCell ref="J71:J72"/>
     <mergeCell ref="E44:E46"/>
     <mergeCell ref="K53:K54"/>
     <mergeCell ref="F57:F58"/>
@@ -4605,12 +4830,14 @@
     <mergeCell ref="M53:M54"/>
     <mergeCell ref="M47:M48"/>
     <mergeCell ref="J8:J9"/>
+    <mergeCell ref="J38:J41"/>
     <mergeCell ref="K55:K56"/>
     <mergeCell ref="B26:B27"/>
-    <mergeCell ref="J38:J41"/>
     <mergeCell ref="E14:E15"/>
     <mergeCell ref="O4:O5"/>
     <mergeCell ref="L18:L19"/>
+    <mergeCell ref="I71:I72"/>
+    <mergeCell ref="K71:K72"/>
     <mergeCell ref="F44:F46"/>
     <mergeCell ref="P36:P37"/>
     <mergeCell ref="K2:K3"/>
@@ -4639,6 +4866,8 @@
     <mergeCell ref="J18:J19"/>
     <mergeCell ref="M30:M33"/>
     <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L69:L70"/>
+    <mergeCell ref="N69:N70"/>
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="I38:I41"/>
     <mergeCell ref="K38:K41"/>
@@ -4673,9 +4902,12 @@
     <mergeCell ref="E36:E37"/>
     <mergeCell ref="A47:A48"/>
     <mergeCell ref="N65:N66"/>
+    <mergeCell ref="I69:I70"/>
+    <mergeCell ref="K69:K70"/>
     <mergeCell ref="O14:O15"/>
     <mergeCell ref="O28:O29"/>
     <mergeCell ref="B59:B60"/>
+    <mergeCell ref="Q71:Q72"/>
     <mergeCell ref="L44:L46"/>
     <mergeCell ref="N44:N46"/>
     <mergeCell ref="B61:B62"/>
@@ -4691,12 +4923,14 @@
     <mergeCell ref="C57:C58"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="H47:H48"/>
+    <mergeCell ref="P71:P72"/>
     <mergeCell ref="J47:J48"/>
     <mergeCell ref="I42:I43"/>
     <mergeCell ref="K42:K43"/>
     <mergeCell ref="K44:K46"/>
     <mergeCell ref="J22:J23"/>
     <mergeCell ref="A53:A54"/>
+    <mergeCell ref="C69:C70"/>
     <mergeCell ref="J51:J52"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="K6:K7"/>
@@ -4717,9 +4951,11 @@
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="B67:B68"/>
     <mergeCell ref="M65:M66"/>
+    <mergeCell ref="H69:H70"/>
     <mergeCell ref="J20:J21"/>
     <mergeCell ref="O65:O66"/>
     <mergeCell ref="L20:L21"/>
+    <mergeCell ref="B69:B70"/>
     <mergeCell ref="G63:G64"/>
     <mergeCell ref="L22:L23"/>
     <mergeCell ref="L34:L35"/>
@@ -4757,14 +4993,17 @@
     <mergeCell ref="J67:J68"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="J61:J62"/>
+    <mergeCell ref="G71:G72"/>
     <mergeCell ref="L61:L62"/>
     <mergeCell ref="B44:B46"/>
     <mergeCell ref="K16:K17"/>
     <mergeCell ref="L36:L37"/>
+    <mergeCell ref="P69:P70"/>
     <mergeCell ref="N36:N37"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="A67:A68"/>
     <mergeCell ref="I2:I3"/>
+    <mergeCell ref="A69:A70"/>
     <mergeCell ref="I22:I23"/>
     <mergeCell ref="K22:K23"/>
     <mergeCell ref="M22:M23"/>
@@ -4792,6 +5031,7 @@
     <mergeCell ref="E8:E9"/>
     <mergeCell ref="I30:I33"/>
     <mergeCell ref="G8:G9"/>
+    <mergeCell ref="J69:J70"/>
     <mergeCell ref="P6:P7"/>
     <mergeCell ref="E38:E41"/>
     <mergeCell ref="F55:F56"/>
@@ -4807,6 +5047,7 @@
     <mergeCell ref="B28:B29"/>
     <mergeCell ref="G18:G19"/>
     <mergeCell ref="I67:I68"/>
+    <mergeCell ref="F71:F72"/>
     <mergeCell ref="K61:K62"/>
     <mergeCell ref="G51:G52"/>
     <mergeCell ref="M61:M62"/>
@@ -4827,6 +5068,7 @@
     <mergeCell ref="A65:A66"/>
     <mergeCell ref="C65:C66"/>
     <mergeCell ref="M28:M29"/>
+    <mergeCell ref="O71:O72"/>
     <mergeCell ref="H44:H46"/>
     <mergeCell ref="J44:J46"/>
     <mergeCell ref="P53:P54"/>
@@ -4846,6 +5088,7 @@
     <mergeCell ref="N63:N64"/>
     <mergeCell ref="P63:P64"/>
     <mergeCell ref="O18:O19"/>
+    <mergeCell ref="L71:L72"/>
     <mergeCell ref="E42:E43"/>
     <mergeCell ref="G42:G43"/>
     <mergeCell ref="J65:J66"/>
@@ -4865,21 +5108,23 @@
     <mergeCell ref="I65:I66"/>
     <mergeCell ref="K65:K66"/>
     <mergeCell ref="N55:N56"/>
+    <mergeCell ref="P55:P56"/>
     <mergeCell ref="H20:H21"/>
     <mergeCell ref="O38:O41"/>
-    <mergeCell ref="P55:P56"/>
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="O24:O25"/>
     <mergeCell ref="J28:J29"/>
     <mergeCell ref="L28:L29"/>
     <mergeCell ref="O16:O17"/>
     <mergeCell ref="Q67:Q68"/>
+    <mergeCell ref="N71:N72"/>
     <mergeCell ref="G44:G46"/>
     <mergeCell ref="O26:O27"/>
     <mergeCell ref="I44:I46"/>
     <mergeCell ref="Q51:Q52"/>
     <mergeCell ref="L8:L9"/>
     <mergeCell ref="N8:N9"/>
+    <mergeCell ref="Q69:Q70"/>
     <mergeCell ref="P8:P9"/>
     <mergeCell ref="B24:B25"/>
     <mergeCell ref="G20:G21"/>
@@ -4891,6 +5136,7 @@
     <mergeCell ref="O42:O43"/>
     <mergeCell ref="C53:C54"/>
     <mergeCell ref="E47:E48"/>
+    <mergeCell ref="M71:M72"/>
     <mergeCell ref="G47:G48"/>
     <mergeCell ref="E22:E23"/>
     <mergeCell ref="N51:N52"/>
@@ -4908,7 +5154,9 @@
     <mergeCell ref="N67:N68"/>
     <mergeCell ref="N61:N62"/>
     <mergeCell ref="P67:P68"/>
+    <mergeCell ref="A71:A72"/>
     <mergeCell ref="P61:P62"/>
+    <mergeCell ref="C71:C72"/>
     <mergeCell ref="H61:H62"/>
     <mergeCell ref="F26:F27"/>
     <mergeCell ref="H36:H37"/>
@@ -4961,14 +5209,18 @@
     <mergeCell ref="H4:H5"/>
     <mergeCell ref="M67:M68"/>
     <mergeCell ref="G67:G68"/>
+    <mergeCell ref="B71:B72"/>
     <mergeCell ref="G61:G62"/>
     <mergeCell ref="I61:I62"/>
     <mergeCell ref="P65:P66"/>
     <mergeCell ref="I36:I37"/>
     <mergeCell ref="B8:B9"/>
+    <mergeCell ref="M69:M70"/>
     <mergeCell ref="A36:A37"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="O20:O21"/>
+    <mergeCell ref="G69:G70"/>
+    <mergeCell ref="O69:O70"/>
     <mergeCell ref="H57:H58"/>
     <mergeCell ref="P44:P46"/>
     <mergeCell ref="E16:E17"/>
@@ -4995,6 +5247,7 @@
     <mergeCell ref="J63:J64"/>
     <mergeCell ref="Q59:Q60"/>
     <mergeCell ref="L63:L64"/>
+    <mergeCell ref="H71:H72"/>
     <mergeCell ref="G30:G33"/>
     <mergeCell ref="A42:A43"/>
     <mergeCell ref="G4:G5"/>
@@ -5007,6 +5260,7 @@
     <mergeCell ref="N20:N21"/>
     <mergeCell ref="K24:K25"/>
     <mergeCell ref="P20:P21"/>
+    <mergeCell ref="F69:F70"/>
     <mergeCell ref="E24:E25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5019,7 +5273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" style="27" min="1" max="2"/>
@@ -5038,7 +5292,7 @@
     <row r="1">
       <c r="A1" s="49" t="inlineStr">
         <is>
-          <t>KPI REPORT | GENERATED: 2026-06-10 18:27 | TOTAL ALL-TIME PRODUCTION: 13542</t>
+          <t>KPI REPORT | GENERATED: 2026-06-11 20:44 | TOTAL ALL-TIME PRODUCTION: 23542</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5300,7 @@
     <row r="4" ht="20.25" customHeight="1" s="27">
       <c r="A4" s="50" t="inlineStr">
         <is>
-          <t>PRODUCTION DATE: 2026-06-10   |   TOTAL DAILY OUTPUT: 9940</t>
+          <t>PRODUCTION DATE: 2026-06-11   |   TOTAL DAILY OUTPUT: 10000</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5353,7 @@
         </is>
       </c>
       <c r="B6" s="53" t="n">
-        <v>9672</v>
+        <v>10000</v>
       </c>
       <c r="D6" s="52" t="inlineStr">
         <is>
@@ -5107,114 +5361,66 @@
         </is>
       </c>
       <c r="E6" s="53" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G6" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10003-X-SUB</t>
+        </is>
+      </c>
+      <c r="H6" s="53" t="n">
         <v>5000</v>
       </c>
-      <c r="G6" s="52" t="inlineStr">
-        <is>
-          <t>MOCK-A01-10003-X-SUB</t>
-        </is>
-      </c>
-      <c r="H6" s="53" t="n">
-        <v>5890</v>
-      </c>
       <c r="J6" s="52" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
       <c r="K6" s="53" t="n">
-        <v>8190</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1" s="27">
-      <c r="A7" s="52" t="inlineStr">
-        <is>
-          <t>Shift B</t>
-        </is>
-      </c>
-      <c r="B7" s="53" t="n">
-        <v>268</v>
-      </c>
-      <c r="D7" s="52" t="inlineStr">
-        <is>
-          <t>333</t>
-        </is>
-      </c>
-      <c r="E7" s="53" t="n">
-        <v>1750</v>
-      </c>
+      <c r="A7" s="52" t="inlineStr"/>
+      <c r="B7" s="52" t="inlineStr"/>
+      <c r="D7" s="54" t="inlineStr"/>
+      <c r="E7" s="54" t="inlineStr"/>
       <c r="G7" s="52" t="inlineStr">
         <is>
-          <t>MOCK-B02-20005-X-SUB</t>
+          <t>MOCK-F06-60001-X-SUB</t>
         </is>
       </c>
       <c r="H7" s="53" t="n">
-        <v>1750</v>
-      </c>
-      <c r="J7" s="52" t="inlineStr">
-        <is>
-          <t>S07</t>
-        </is>
-      </c>
-      <c r="K7" s="53" t="n">
-        <v>1750</v>
-      </c>
+        <v>5000</v>
+      </c>
+      <c r="J7" s="54" t="inlineStr"/>
+      <c r="K7" s="54" t="inlineStr"/>
     </row>
     <row r="8" ht="16.5" customHeight="1" s="27">
       <c r="A8" s="52" t="inlineStr"/>
       <c r="B8" s="52" t="inlineStr"/>
-      <c r="D8" s="52" t="inlineStr">
-        <is>
-          <t>5566</t>
-        </is>
-      </c>
-      <c r="E8" s="53" t="n">
-        <v>1400</v>
-      </c>
-      <c r="G8" s="52" t="inlineStr">
-        <is>
-          <t>MOCK-E05-50003-X-SUB</t>
-        </is>
-      </c>
-      <c r="H8" s="53" t="n">
-        <v>1400</v>
-      </c>
+      <c r="D8" s="54" t="inlineStr"/>
+      <c r="E8" s="54" t="inlineStr"/>
+      <c r="G8" s="54" t="inlineStr"/>
+      <c r="H8" s="54" t="inlineStr"/>
       <c r="J8" s="54" t="inlineStr"/>
       <c r="K8" s="54" t="inlineStr"/>
     </row>
     <row r="9" ht="16.5" customHeight="1" s="27">
       <c r="A9" s="52" t="inlineStr"/>
       <c r="B9" s="52" t="inlineStr"/>
-      <c r="D9" s="52" t="inlineStr">
-        <is>
-          <t>677</t>
-        </is>
-      </c>
-      <c r="E9" s="53" t="n">
-        <v>900</v>
-      </c>
-      <c r="G9" s="52" t="inlineStr">
-        <is>
-          <t>MOCK-A01-10001-X-SUB</t>
-        </is>
-      </c>
-      <c r="H9" s="53" t="n">
-        <v>900</v>
-      </c>
+      <c r="D9" s="54" t="inlineStr"/>
+      <c r="E9" s="54" t="inlineStr"/>
+      <c r="G9" s="54" t="inlineStr"/>
+      <c r="H9" s="54" t="inlineStr"/>
       <c r="J9" s="54" t="inlineStr"/>
       <c r="K9" s="54" t="inlineStr"/>
     </row>
     <row r="10" ht="16.5" customHeight="1" s="27">
       <c r="A10" s="52" t="inlineStr"/>
       <c r="B10" s="52" t="inlineStr"/>
-      <c r="D10" s="52" t="inlineStr">
-        <is>
-          <t>666</t>
-        </is>
-      </c>
-      <c r="E10" s="53" t="n">
-        <v>890</v>
-      </c>
+      <c r="D10" s="54" t="inlineStr"/>
+      <c r="E10" s="54" t="inlineStr"/>
       <c r="G10" s="54" t="inlineStr"/>
       <c r="H10" s="54" t="inlineStr"/>
       <c r="J10" s="54" t="inlineStr"/>
@@ -5223,7 +5429,7 @@
     <row r="12" ht="20.25" customHeight="1" s="27">
       <c r="A12" s="50" t="inlineStr">
         <is>
-          <t>PRODUCTION DATE: 2026-06-09   |   TOTAL DAILY OUTPUT: 1384</t>
+          <t>PRODUCTION DATE: 2026-06-10   |   TOTAL DAILY OUTPUT: 9940</t>
         </is>
       </c>
     </row>
@@ -5276,57 +5482,57 @@
         </is>
       </c>
       <c r="B14" s="53" t="n">
-        <v>1254</v>
+        <v>9672</v>
       </c>
       <c r="D14" s="52" t="inlineStr">
         <is>
-          <t>778</t>
+          <t>111</t>
         </is>
       </c>
       <c r="E14" s="53" t="n">
-        <v>900</v>
+        <v>5000</v>
       </c>
       <c r="G14" s="52" t="inlineStr">
         <is>
-          <t>MOCK-B02-20001-X-SUB</t>
+          <t>MOCK-A01-10003-X-SUB</t>
         </is>
       </c>
       <c r="H14" s="53" t="n">
-        <v>900</v>
+        <v>5890</v>
       </c>
       <c r="J14" s="52" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S06</t>
         </is>
       </c>
       <c r="K14" s="53" t="n">
-        <v>900</v>
+        <v>8190</v>
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1" s="27">
       <c r="A15" s="52" t="inlineStr">
         <is>
-          <t>Shift C</t>
+          <t>Shift B</t>
         </is>
       </c>
       <c r="B15" s="53" t="n">
-        <v>130</v>
+        <v>268</v>
       </c>
       <c r="D15" s="52" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>333</t>
         </is>
       </c>
       <c r="E15" s="53" t="n">
-        <v>260</v>
+        <v>1750</v>
       </c>
       <c r="G15" s="52" t="inlineStr">
         <is>
-          <t>MOCK-E05-50003-X-SUB</t>
+          <t>MOCK-B02-20005-X-SUB</t>
         </is>
       </c>
       <c r="H15" s="53" t="n">
-        <v>134</v>
+        <v>1750</v>
       </c>
       <c r="J15" s="52" t="inlineStr">
         <is>
@@ -5334,7 +5540,7 @@
         </is>
       </c>
       <c r="K15" s="53" t="n">
-        <v>260</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="27">
@@ -5342,47 +5548,41 @@
       <c r="B16" s="52" t="inlineStr"/>
       <c r="D16" s="52" t="inlineStr">
         <is>
-          <t>771</t>
+          <t>5566</t>
         </is>
       </c>
       <c r="E16" s="53" t="n">
-        <v>134</v>
+        <v>1400</v>
       </c>
       <c r="G16" s="52" t="inlineStr">
         <is>
-          <t>MOCK-A01-10006-X-SUB</t>
+          <t>MOCK-E05-50003-X-SUB</t>
         </is>
       </c>
       <c r="H16" s="53" t="n">
-        <v>130</v>
-      </c>
-      <c r="J16" s="52" t="inlineStr">
-        <is>
-          <t>S11</t>
-        </is>
-      </c>
-      <c r="K16" s="53" t="n">
-        <v>224</v>
-      </c>
+        <v>1400</v>
+      </c>
+      <c r="J16" s="54" t="inlineStr"/>
+      <c r="K16" s="54" t="inlineStr"/>
     </row>
     <row r="17" ht="16.5" customHeight="1" s="27">
       <c r="A17" s="52" t="inlineStr"/>
       <c r="B17" s="52" t="inlineStr"/>
       <c r="D17" s="52" t="inlineStr">
         <is>
-          <t>770</t>
+          <t>677</t>
         </is>
       </c>
       <c r="E17" s="53" t="n">
-        <v>90</v>
+        <v>900</v>
       </c>
       <c r="G17" s="52" t="inlineStr">
         <is>
-          <t>MOCK-F06-60001-X-SUB</t>
+          <t>MOCK-A01-10001-X-SUB</t>
         </is>
       </c>
       <c r="H17" s="53" t="n">
-        <v>130</v>
+        <v>900</v>
       </c>
       <c r="J17" s="54" t="inlineStr"/>
       <c r="K17" s="54" t="inlineStr"/>
@@ -5390,23 +5590,23 @@
     <row r="18" ht="16.5" customHeight="1" s="27">
       <c r="A18" s="52" t="inlineStr"/>
       <c r="B18" s="52" t="inlineStr"/>
-      <c r="D18" s="54" t="inlineStr"/>
-      <c r="E18" s="54" t="inlineStr"/>
-      <c r="G18" s="52" t="inlineStr">
-        <is>
-          <t>MOCK-C03-30006-X-SUB</t>
-        </is>
-      </c>
-      <c r="H18" s="53" t="n">
-        <v>90</v>
-      </c>
+      <c r="D18" s="52" t="inlineStr">
+        <is>
+          <t>666</t>
+        </is>
+      </c>
+      <c r="E18" s="53" t="n">
+        <v>890</v>
+      </c>
+      <c r="G18" s="54" t="inlineStr"/>
+      <c r="H18" s="54" t="inlineStr"/>
       <c r="J18" s="54" t="inlineStr"/>
       <c r="K18" s="54" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="50" t="inlineStr">
         <is>
-          <t>PRODUCTION DATE: 2026-06-08   |   TOTAL DAILY OUTPUT: 2218</t>
+          <t>PRODUCTION DATE: 2026-06-09   |   TOTAL DAILY OUTPUT: 1384</t>
         </is>
       </c>
     </row>
@@ -5459,7 +5659,7 @@
         </is>
       </c>
       <c r="B22" s="53" t="n">
-        <v>1975</v>
+        <v>1254</v>
       </c>
       <c r="D22" s="52" t="inlineStr">
         <is>
@@ -5467,15 +5667,15 @@
         </is>
       </c>
       <c r="E22" s="53" t="n">
-        <v>1164</v>
+        <v>900</v>
       </c>
       <c r="G22" s="52" t="inlineStr">
         <is>
-          <t>MOCK-G07-70001-X-SUB</t>
+          <t>MOCK-B02-20001-X-SUB</t>
         </is>
       </c>
       <c r="H22" s="53" t="n">
-        <v>922</v>
+        <v>900</v>
       </c>
       <c r="J22" s="52" t="inlineStr">
         <is>
@@ -5483,33 +5683,33 @@
         </is>
       </c>
       <c r="K22" s="53" t="n">
-        <v>1164</v>
+        <v>900</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="52" t="inlineStr">
         <is>
-          <t>Shift B</t>
+          <t>Shift C</t>
         </is>
       </c>
       <c r="B23" s="53" t="n">
-        <v>243</v>
+        <v>130</v>
       </c>
       <c r="D23" s="52" t="inlineStr">
         <is>
-          <t>777</t>
+          <t>543</t>
         </is>
       </c>
       <c r="E23" s="53" t="n">
-        <v>333</v>
+        <v>260</v>
       </c>
       <c r="G23" s="52" t="inlineStr">
         <is>
-          <t>MOCK-A01-10001-X-SUB</t>
+          <t>MOCK-E05-50003-X-SUB</t>
         </is>
       </c>
       <c r="H23" s="53" t="n">
-        <v>752</v>
+        <v>134</v>
       </c>
       <c r="J23" s="52" t="inlineStr">
         <is>
@@ -5517,7 +5717,7 @@
         </is>
       </c>
       <c r="K23" s="53" t="n">
-        <v>646</v>
+        <v>260</v>
       </c>
     </row>
     <row r="24">
@@ -5525,27 +5725,27 @@
       <c r="B24" s="52" t="inlineStr"/>
       <c r="D24" s="52" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>771</t>
         </is>
       </c>
       <c r="E24" s="53" t="n">
-        <v>234</v>
+        <v>134</v>
       </c>
       <c r="G24" s="52" t="inlineStr">
         <is>
-          <t>MOCK-E05-50003-X-SUB</t>
+          <t>MOCK-A01-10006-X-SUB</t>
         </is>
       </c>
       <c r="H24" s="53" t="n">
-        <v>256</v>
+        <v>130</v>
       </c>
       <c r="J24" s="52" t="inlineStr">
         <is>
-          <t>S06</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="K24" s="53" t="n">
-        <v>408</v>
+        <v>224</v>
       </c>
     </row>
     <row r="25">
@@ -5553,19 +5753,19 @@
       <c r="B25" s="52" t="inlineStr"/>
       <c r="D25" s="52" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>770</t>
         </is>
       </c>
       <c r="E25" s="53" t="n">
-        <v>123</v>
+        <v>90</v>
       </c>
       <c r="G25" s="52" t="inlineStr">
         <is>
-          <t>MOCK-B02-20004-X-SUB</t>
+          <t>MOCK-F06-60001-X-SUB</t>
         </is>
       </c>
       <c r="H25" s="53" t="n">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="J25" s="54" t="inlineStr"/>
       <c r="K25" s="54" t="inlineStr"/>
@@ -5573,31 +5773,215 @@
     <row r="26">
       <c r="A26" s="52" t="inlineStr"/>
       <c r="B26" s="52" t="inlineStr"/>
-      <c r="D26" s="52" t="inlineStr">
-        <is>
-          <t>888</t>
-        </is>
-      </c>
-      <c r="E26" s="53" t="n">
-        <v>120</v>
-      </c>
+      <c r="D26" s="54" t="inlineStr"/>
+      <c r="E26" s="54" t="inlineStr"/>
       <c r="G26" s="52" t="inlineStr">
         <is>
-          <t>MOCK-A01-10003-X-SUB</t>
+          <t>MOCK-C03-30006-X-SUB</t>
         </is>
       </c>
       <c r="H26" s="53" t="n">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="J26" s="54" t="inlineStr"/>
       <c r="K26" s="54" t="inlineStr"/>
     </row>
+    <row r="28">
+      <c r="A28" s="50" t="inlineStr">
+        <is>
+          <t>PRODUCTION DATE: 2026-06-08   |   TOTAL DAILY OUTPUT: 2218</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="51" t="inlineStr">
+        <is>
+          <t>SHIFT</t>
+        </is>
+      </c>
+      <c r="B29" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="D29" s="51" t="inlineStr">
+        <is>
+          <t>TOP 5 OPERATORS</t>
+        </is>
+      </c>
+      <c r="E29" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="G29" s="51" t="inlineStr">
+        <is>
+          <t>TOP 5 PRODUCTS</t>
+        </is>
+      </c>
+      <c r="H29" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="J29" s="51" t="inlineStr">
+        <is>
+          <t>STATIONS</t>
+        </is>
+      </c>
+      <c r="K29" s="51" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="52" t="inlineStr">
+        <is>
+          <t>Shift A</t>
+        </is>
+      </c>
+      <c r="B30" s="53" t="n">
+        <v>1975</v>
+      </c>
+      <c r="D30" s="52" t="inlineStr">
+        <is>
+          <t>778</t>
+        </is>
+      </c>
+      <c r="E30" s="53" t="n">
+        <v>1164</v>
+      </c>
+      <c r="G30" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-G07-70001-X-SUB</t>
+        </is>
+      </c>
+      <c r="H30" s="53" t="n">
+        <v>922</v>
+      </c>
+      <c r="J30" s="52" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="K30" s="53" t="n">
+        <v>1164</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="52" t="inlineStr">
+        <is>
+          <t>Shift B</t>
+        </is>
+      </c>
+      <c r="B31" s="53" t="n">
+        <v>243</v>
+      </c>
+      <c r="D31" s="52" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="E31" s="53" t="n">
+        <v>333</v>
+      </c>
+      <c r="G31" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10001-X-SUB</t>
+        </is>
+      </c>
+      <c r="H31" s="53" t="n">
+        <v>752</v>
+      </c>
+      <c r="J31" s="52" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="K31" s="53" t="n">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="52" t="inlineStr"/>
+      <c r="B32" s="52" t="inlineStr"/>
+      <c r="D32" s="52" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="E32" s="53" t="n">
+        <v>234</v>
+      </c>
+      <c r="G32" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-E05-50003-X-SUB</t>
+        </is>
+      </c>
+      <c r="H32" s="53" t="n">
+        <v>256</v>
+      </c>
+      <c r="J32" s="52" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="K32" s="53" t="n">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="52" t="inlineStr"/>
+      <c r="B33" s="52" t="inlineStr"/>
+      <c r="D33" s="52" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="E33" s="53" t="n">
+        <v>123</v>
+      </c>
+      <c r="G33" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-B02-20004-X-SUB</t>
+        </is>
+      </c>
+      <c r="H33" s="53" t="n">
+        <v>220</v>
+      </c>
+      <c r="J33" s="54" t="inlineStr"/>
+      <c r="K33" s="54" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="52" t="inlineStr"/>
+      <c r="B34" s="52" t="inlineStr"/>
+      <c r="D34" s="52" t="inlineStr">
+        <is>
+          <t>888</t>
+        </is>
+      </c>
+      <c r="E34" s="53" t="n">
+        <v>120</v>
+      </c>
+      <c r="G34" s="52" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10003-X-SUB</t>
+        </is>
+      </c>
+      <c r="H34" s="53" t="n">
+        <v>68</v>
+      </c>
+      <c r="J34" s="54" t="inlineStr"/>
+      <c r="K34" s="54" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:K2"/>
+  <mergeCells count="5">
     <mergeCell ref="A12:K12"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A28:K28"/>
+    <mergeCell ref="A1:K2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add test suite, report generation logic, and PyInstaller build configuration for Quality App
</commit_message>
<xml_diff>
--- a/data/production_data.xlsx
+++ b/data/production_data.xlsx
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -577,7 +577,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>KPI REPORT | GENERATED: 2026-06-13 16:17 | TOTAL ALL-TIME PRODUCTION: 250</t>
+          <t>KPI REPORT | GENERATED: 2026-06-14 16:26 | TOTAL ALL-TIME PRODUCTION: 720</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>PRODUCTION DATE: 2026-06-13  |  TOTAL DAILY OUTPUT: 250</t>
+          <t>PRODUCTION DATE: 2026-06-14  |  TOTAL DAILY OUTPUT: 300</t>
         </is>
       </c>
     </row>
@@ -648,23 +648,23 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>140</v>
+        <v>300</v>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>777</t>
         </is>
       </c>
       <c r="E6" s="9" t="n">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>TEST1</t>
+          <t>MOCK-A01-10004-X-SUB</t>
         </is>
       </c>
       <c r="H6" s="9" t="n">
-        <v>160</v>
+        <v>300</v>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
@@ -672,42 +672,18 @@
         </is>
       </c>
       <c r="K6" s="9" t="n">
-        <v>250</v>
-      </c>
-      <c r="M6" s="8" t="inlineStr">
-        <is>
-          <t>543 (Deplacement,Quality )</t>
-        </is>
-      </c>
-      <c r="N6" s="9" t="n">
-        <v>57</v>
-      </c>
+        <v>300</v>
+      </c>
+      <c r="M6" s="10" t="inlineStr"/>
+      <c r="N6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Shift B</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n">
-        <v>110</v>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>544</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>TEST2</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>80</v>
-      </c>
+      <c r="A7" s="8" t="inlineStr"/>
+      <c r="B7" s="8" t="inlineStr"/>
+      <c r="D7" s="10" t="inlineStr"/>
+      <c r="E7" s="10" t="inlineStr"/>
+      <c r="G7" s="10" t="inlineStr"/>
+      <c r="H7" s="10" t="inlineStr"/>
       <c r="J7" s="10" t="inlineStr"/>
       <c r="K7" s="10" t="inlineStr"/>
       <c r="M7" s="10" t="inlineStr"/>
@@ -718,14 +694,8 @@
       <c r="B8" s="8" t="inlineStr"/>
       <c r="D8" s="10" t="inlineStr"/>
       <c r="E8" s="10" t="inlineStr"/>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>MOCK-D04-40001-X-SUB</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>10</v>
-      </c>
+      <c r="G8" s="10" t="inlineStr"/>
+      <c r="H8" s="10" t="inlineStr"/>
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
       <c r="M8" s="10" t="inlineStr"/>
@@ -755,8 +725,182 @@
       <c r="M10" s="10" t="inlineStr"/>
       <c r="N10" s="10" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>PRODUCTION DATE: 2026-06-13  |  TOTAL DAILY OUTPUT: 250</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>SHIFT</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>TOP 5 OPERATORS</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>TOP 5 PRODUCTS</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>STATIONS</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>OUTPUT</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>DOWNTIME (OP)</t>
+        </is>
+      </c>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>MINS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Shift A</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>543</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>220</v>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>TEST1</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>160</v>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="M14" s="8" t="inlineStr">
+        <is>
+          <t>543 (Deplacement,Quality )</t>
+        </is>
+      </c>
+      <c r="N14" s="9" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Shift B</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>110</v>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>544</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>TEST2</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="J15" s="10" t="inlineStr"/>
+      <c r="K15" s="10" t="inlineStr"/>
+      <c r="M15" s="10" t="inlineStr"/>
+      <c r="N15" s="10" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr"/>
+      <c r="B16" s="8" t="inlineStr"/>
+      <c r="D16" s="10" t="inlineStr"/>
+      <c r="E16" s="10" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>MOCK-D04-40001-X-SUB</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="J16" s="10" t="inlineStr"/>
+      <c r="K16" s="10" t="inlineStr"/>
+      <c r="M16" s="10" t="inlineStr"/>
+      <c r="N16" s="10" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr"/>
+      <c r="B17" s="8" t="inlineStr"/>
+      <c r="D17" s="10" t="inlineStr"/>
+      <c r="E17" s="10" t="inlineStr"/>
+      <c r="G17" s="10" t="inlineStr"/>
+      <c r="H17" s="10" t="inlineStr"/>
+      <c r="J17" s="10" t="inlineStr"/>
+      <c r="K17" s="10" t="inlineStr"/>
+      <c r="M17" s="10" t="inlineStr"/>
+      <c r="N17" s="10" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr"/>
+      <c r="B18" s="8" t="inlineStr"/>
+      <c r="D18" s="10" t="inlineStr"/>
+      <c r="E18" s="10" t="inlineStr"/>
+      <c r="G18" s="10" t="inlineStr"/>
+      <c r="H18" s="10" t="inlineStr"/>
+      <c r="J18" s="10" t="inlineStr"/>
+      <c r="K18" s="10" t="inlineStr"/>
+      <c r="M18" s="10" t="inlineStr"/>
+      <c r="N18" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A12:N12"/>
     <mergeCell ref="A1:N2"/>
     <mergeCell ref="A4:N4"/>
   </mergeCells>
@@ -770,7 +914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q21"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2390,12 +2534,12 @@
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-06-14 16:29</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>A</t>
         </is>
       </c>
       <c r="P19" s="4" t="inlineStr">
@@ -2463,23 +2607,150 @@
       <c r="P21" s="12" t="n"/>
       <c r="Q21" s="12" t="n"/>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>SB202606141626S06A01927E</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10004-X-SUB</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Alpha Subsystem Left</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10004-Y-PRT</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Alpha Core Left</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>RRRR</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>777</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-14 16:26</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n"/>
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>MOCK-A01-10005-Z-PRT</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Alpha Buffer Left</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="12" t="n"/>
+      <c r="J23" s="12" t="n"/>
+      <c r="K23" s="12" t="n"/>
+      <c r="L23" s="12" t="n"/>
+      <c r="M23" s="12" t="n"/>
+      <c r="N23" s="12" t="n"/>
+      <c r="O23" s="12" t="n"/>
+      <c r="P23" s="12" t="n"/>
+      <c r="Q23" s="12" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="J19:J21"/>
+  <mergeCells count="30">
+    <mergeCell ref="N22:N23"/>
+    <mergeCell ref="P22:P23"/>
+    <mergeCell ref="N19:N21"/>
+    <mergeCell ref="P19:P21"/>
+    <mergeCell ref="H19:H21"/>
+    <mergeCell ref="I19:I21"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="M22:M23"/>
+    <mergeCell ref="Q22:Q23"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="H22:H23"/>
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="K19:K21"/>
     <mergeCell ref="M19:M21"/>
     <mergeCell ref="C19:C21"/>
-    <mergeCell ref="N19:N21"/>
+    <mergeCell ref="O19:O21"/>
+    <mergeCell ref="F19:F21"/>
+    <mergeCell ref="O22:O23"/>
+    <mergeCell ref="L22:L23"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="J19:J21"/>
+    <mergeCell ref="L19:L21"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="Q19:Q21"/>
     <mergeCell ref="G19:G21"/>
-    <mergeCell ref="O19:O21"/>
     <mergeCell ref="B19:B21"/>
-    <mergeCell ref="H19:H21"/>
-    <mergeCell ref="F19:F21"/>
-    <mergeCell ref="L19:L21"/>
-    <mergeCell ref="I19:I21"/>
-    <mergeCell ref="P19:P21"/>
-    <mergeCell ref="Q19:Q21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>